<commit_message>
feat(epirank): update 原_Germany daytime results, remove duplicate reverse files
</commit_message>
<xml_diff>
--- a/EpiRank_原_Germany/ERA_result_d_0.95_daytime_0.5_loops_110.xlsx
+++ b/EpiRank_原_Germany/ERA_result_d_0.95_daytime_0.5_loops_110.xlsx
@@ -859,10 +859,10 @@
         <v>0.019464</v>
       </c>
       <c r="Y3" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z3" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA3" s="3" t="n">
         <v>34035</v>
@@ -1435,10 +1435,10 @@
         <v>0.01118</v>
       </c>
       <c r="Y7" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z7" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA7" s="3" t="n">
         <v>6805</v>
@@ -2293,10 +2293,10 @@
         <v>0.005667</v>
       </c>
       <c r="Y13" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z13" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA13" s="3" t="n">
         <v>1620</v>
@@ -2558,10 +2558,10 @@
         <v>0.005871</v>
       </c>
       <c r="Y15" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z15" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA15" s="3" t="n">
         <v>4465</v>
@@ -3058,10 +3058,10 @@
         <v>0.004867</v>
       </c>
       <c r="Y19" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z19" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA19" s="3" t="n">
         <v>6813</v>
@@ -3418,10 +3418,10 @@
         <v>0.004559</v>
       </c>
       <c r="Y22" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z22" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA22" s="3" t="n">
         <v>4123</v>
@@ -4018,10 +4018,10 @@
         <v>0.004805</v>
       </c>
       <c r="Y27" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z27" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA27" s="3" t="n">
         <v>1432</v>
@@ -4138,10 +4138,10 @@
         <v>0.004224</v>
       </c>
       <c r="Y28" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z28" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA28" s="3" t="n">
         <v>3369</v>
@@ -4258,10 +4258,10 @@
         <v>0.003699</v>
       </c>
       <c r="Y29" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z29" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA29" s="3" t="n">
         <v>2262</v>
@@ -4378,10 +4378,10 @@
         <v>0.004758</v>
       </c>
       <c r="Y30" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z30" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA30" s="3" t="n">
         <v>2551</v>
@@ -4738,10 +4738,10 @@
         <v>0.003686</v>
       </c>
       <c r="Y33" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z33" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA33" s="3" t="n">
         <v>3059</v>
@@ -5098,10 +5098,10 @@
         <v>0.003865</v>
       </c>
       <c r="Y36" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z36" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA36" s="3" t="n">
         <v>11679</v>
@@ -5218,7 +5218,7 @@
         <v>0.003682</v>
       </c>
       <c r="Y37" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z37" s="3" t="n">
         <v>-0</v>
@@ -5578,7 +5578,7 @@
         <v>0.003994</v>
       </c>
       <c r="Y40" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z40" s="3" t="n">
         <v>0</v>
@@ -5818,10 +5818,10 @@
         <v>0.003867</v>
       </c>
       <c r="Y42" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z42" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA42" s="3" t="n">
         <v>3417</v>
@@ -6058,10 +6058,10 @@
         <v>0.003516</v>
       </c>
       <c r="Y44" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z44" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA44" s="3" t="n">
         <v>2752</v>
@@ -6298,10 +6298,10 @@
         <v>0.004055</v>
       </c>
       <c r="Y46" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z46" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA46" s="3" t="n">
         <v>1989</v>
@@ -6661,7 +6661,7 @@
         <v>0</v>
       </c>
       <c r="Z49" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA49" s="3" t="n">
         <v>2526</v>
@@ -7261,7 +7261,7 @@
         <v>0</v>
       </c>
       <c r="Z54" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA54" s="3" t="n">
         <v>930</v>
@@ -7498,7 +7498,7 @@
         <v>0.00306</v>
       </c>
       <c r="Y56" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z56" s="3" t="n">
         <v>-0</v>
@@ -7618,10 +7618,10 @@
         <v>0.003258</v>
       </c>
       <c r="Y57" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z57" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA57" s="3" t="n">
         <v>1293</v>
@@ -7978,10 +7978,10 @@
         <v>0.003378</v>
       </c>
       <c r="Y60" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z60" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA60" s="3" t="n">
         <v>2142</v>
@@ -8338,10 +8338,10 @@
         <v>0.003143</v>
       </c>
       <c r="Y63" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z63" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA63" s="3" t="n">
         <v>2303</v>
@@ -8698,7 +8698,7 @@
         <v>0.002932</v>
       </c>
       <c r="Y66" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z66" s="3" t="n">
         <v>0</v>
@@ -10501,7 +10501,7 @@
         <v>0</v>
       </c>
       <c r="Z81" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA81" s="3" t="n">
         <v>871</v>
@@ -10978,10 +10978,10 @@
         <v>0.002739</v>
       </c>
       <c r="Y85" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z85" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA85" s="3" t="n">
         <v>2843</v>
@@ -11458,10 +11458,10 @@
         <v>0.002894</v>
       </c>
       <c r="Y89" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z89" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA89" s="3" t="n">
         <v>1151</v>
@@ -11698,10 +11698,10 @@
         <v>0.00271</v>
       </c>
       <c r="Y91" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z91" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA91" s="3" t="n">
         <v>2304</v>
@@ -11818,7 +11818,7 @@
         <v>0.003086</v>
       </c>
       <c r="Y92" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z92" s="3" t="n">
         <v>-0</v>
@@ -12058,10 +12058,10 @@
         <v>0.003072</v>
       </c>
       <c r="Y94" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z94" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA94" s="3" t="n">
         <v>1472</v>
@@ -13018,10 +13018,10 @@
         <v>0.003001</v>
       </c>
       <c r="Y102" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z102" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA102" s="3" t="n">
         <v>3835</v>
@@ -13378,10 +13378,10 @@
         <v>0.002646</v>
       </c>
       <c r="Y105" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z105" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA105" s="3" t="n">
         <v>4116</v>
@@ -13501,7 +13501,7 @@
         <v>0</v>
       </c>
       <c r="Z106" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA106" s="3" t="n">
         <v>1871</v>
@@ -13978,10 +13978,10 @@
         <v>0.002646</v>
       </c>
       <c r="Y110" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z110" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA110" s="3" t="n">
         <v>2711</v>
@@ -14701,7 +14701,7 @@
         <v>0</v>
       </c>
       <c r="Z116" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA116" s="3" t="n">
         <v>2287</v>
@@ -15478,10 +15478,10 @@
         <v>0.002324</v>
       </c>
       <c r="Y123" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z123" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA123" s="3" t="n">
         <v>2532</v>
@@ -15591,7 +15591,7 @@
         <v>0</v>
       </c>
       <c r="Z124" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA124" s="3" t="n">
         <v>5101</v>
@@ -15698,10 +15698,10 @@
         <v>0.002932</v>
       </c>
       <c r="Y125" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z125" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA125" s="3" t="n">
         <v>1517</v>
@@ -16581,7 +16581,7 @@
         <v>0</v>
       </c>
       <c r="Z133" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA133" s="3" t="n">
         <v>1776</v>
@@ -16908,10 +16908,10 @@
         <v>0.002515</v>
       </c>
       <c r="Y136" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z136" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA136" s="3" t="n">
         <v>828</v>
@@ -17128,7 +17128,7 @@
         <v>0.002078</v>
       </c>
       <c r="Y138" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z138" s="3" t="n">
         <v>-0</v>
@@ -18118,10 +18118,10 @@
         <v>0.002564</v>
       </c>
       <c r="Y147" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z147" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA147" s="3" t="n">
         <v>2616</v>
@@ -18778,10 +18778,10 @@
         <v>0.00214</v>
       </c>
       <c r="Y153" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z153" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA153" s="3" t="n">
         <v>1559</v>
@@ -19328,10 +19328,10 @@
         <v>0.002328</v>
       </c>
       <c r="Y158" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z158" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA158" s="3" t="n">
         <v>1267</v>
@@ -19551,7 +19551,7 @@
         <v>0</v>
       </c>
       <c r="Z160" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA160" s="3" t="n">
         <v>3546</v>
@@ -19768,7 +19768,7 @@
         <v>0.002184</v>
       </c>
       <c r="Y162" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z162" s="3" t="n">
         <v>-0</v>
@@ -19878,10 +19878,10 @@
         <v>0.002324</v>
       </c>
       <c r="Y163" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z163" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA163" s="3" t="n">
         <v>1662</v>
@@ -20098,7 +20098,7 @@
         <v>0.002271</v>
       </c>
       <c r="Y165" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z165" s="3" t="n">
         <v>0</v>
@@ -20761,7 +20761,7 @@
         <v>0</v>
       </c>
       <c r="Z171" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA171" s="3" t="n">
         <v>1737</v>
@@ -21091,7 +21091,7 @@
         <v>0</v>
       </c>
       <c r="Z174" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA174" s="3" t="n">
         <v>1727</v>
@@ -21308,10 +21308,10 @@
         <v>0.001886</v>
       </c>
       <c r="Y176" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z176" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA176" s="3" t="n">
         <v>1626</v>
@@ -22628,10 +22628,10 @@
         <v>0.002033</v>
       </c>
       <c r="Y188" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z188" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA188" s="3" t="n">
         <v>1846</v>
@@ -22848,10 +22848,10 @@
         <v>0.002054</v>
       </c>
       <c r="Y190" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z190" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA190" s="3" t="n">
         <v>1712</v>
@@ -23068,10 +23068,10 @@
         <v>0.001946</v>
       </c>
       <c r="Y192" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z192" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA192" s="3" t="n">
         <v>1654</v>
@@ -23618,10 +23618,10 @@
         <v>0.002434</v>
       </c>
       <c r="Y197" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z197" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA197" s="3" t="n">
         <v>284</v>
@@ -23951,7 +23951,7 @@
         <v>-0</v>
       </c>
       <c r="Z200" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA200" s="3" t="n">
         <v>1957</v>
@@ -24718,10 +24718,10 @@
         <v>0.001965</v>
       </c>
       <c r="Y207" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z207" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA207" s="3" t="n">
         <v>3507</v>
@@ -24828,7 +24828,7 @@
         <v>0.001861</v>
       </c>
       <c r="Y208" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z208" s="3" t="n">
         <v>-0</v>
@@ -25048,10 +25048,10 @@
         <v>0.002155</v>
       </c>
       <c r="Y210" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z210" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA210" s="3" t="n">
         <v>1407</v>
@@ -25158,10 +25158,10 @@
         <v>0.001842</v>
       </c>
       <c r="Y211" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z211" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA211" s="3" t="n">
         <v>1124</v>
@@ -25268,10 +25268,10 @@
         <v>0.002032</v>
       </c>
       <c r="Y212" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z212" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA212" s="3" t="n">
         <v>1359</v>
@@ -25488,10 +25488,10 @@
         <v>0.001952</v>
       </c>
       <c r="Y214" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z214" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA214" s="3" t="n">
         <v>952</v>
@@ -26368,7 +26368,7 @@
         <v>0.00202</v>
       </c>
       <c r="Y222" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z222" s="3" t="n">
         <v>0</v>
@@ -27248,10 +27248,10 @@
         <v>0.001956</v>
       </c>
       <c r="Y230" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z230" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA230" s="3" t="n">
         <v>2206</v>
@@ -27471,7 +27471,7 @@
         <v>0</v>
       </c>
       <c r="Z232" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA232" s="3" t="n">
         <v>1275</v>
@@ -27688,7 +27688,7 @@
         <v>0.001896</v>
       </c>
       <c r="Y234" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z234" s="3" t="n">
         <v>0</v>
@@ -28348,7 +28348,7 @@
         <v>0.001717</v>
       </c>
       <c r="Y240" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z240" s="3" t="n">
         <v>0</v>
@@ -28568,10 +28568,10 @@
         <v>0.001953</v>
       </c>
       <c r="Y242" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z242" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA242" s="3" t="n">
         <v>1481</v>
@@ -28678,10 +28678,10 @@
         <v>0.00162</v>
       </c>
       <c r="Y243" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z243" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA243" s="3" t="n">
         <v>1538</v>
@@ -28898,10 +28898,10 @@
         <v>0.001919</v>
       </c>
       <c r="Y245" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z245" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA245" s="3" t="n">
         <v>552</v>
@@ -29778,10 +29778,10 @@
         <v>0.001785</v>
       </c>
       <c r="Y253" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z253" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA253" s="3" t="n">
         <v>1929</v>
@@ -30658,7 +30658,7 @@
         <v>0.001586</v>
       </c>
       <c r="Y261" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z261" s="3" t="n">
         <v>0</v>
@@ -31158,10 +31158,10 @@
         <v>0.001815</v>
       </c>
       <c r="Y266" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z266" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA266" s="3" t="n">
         <v>1523</v>
@@ -31561,7 +31561,7 @@
         <v>-0</v>
       </c>
       <c r="Z270" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA270" s="3" t="n">
         <v>692</v>
@@ -31958,10 +31958,10 @@
         <v>0.001683</v>
       </c>
       <c r="Y274" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z274" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA274" s="3" t="n">
         <v>3118</v>
@@ -32158,10 +32158,10 @@
         <v>0.001928</v>
       </c>
       <c r="Y276" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z276" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA276" s="3" t="n">
         <v>348</v>
@@ -32458,10 +32458,10 @@
         <v>0.001623</v>
       </c>
       <c r="Y279" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z279" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA279" s="3" t="n">
         <v>1102</v>
@@ -32558,10 +32558,10 @@
         <v>0.001707</v>
       </c>
       <c r="Y280" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z280" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA280" s="3" t="n">
         <v>745</v>
@@ -32758,7 +32758,7 @@
         <v>0.001666</v>
       </c>
       <c r="Y282" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z282" s="3" t="n">
         <v>0</v>
@@ -33158,10 +33158,10 @@
         <v>0.001605</v>
       </c>
       <c r="Y286" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z286" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA286" s="3" t="n">
         <v>627</v>
@@ -33258,10 +33258,10 @@
         <v>0.00163</v>
       </c>
       <c r="Y287" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z287" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA287" s="3" t="n">
         <v>2337</v>
@@ -33458,10 +33458,10 @@
         <v>0.001646</v>
       </c>
       <c r="Y289" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z289" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA289" s="3" t="n">
         <v>3450</v>
@@ -33758,7 +33758,7 @@
         <v>0.001396</v>
       </c>
       <c r="Y292" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z292" s="3" t="n">
         <v>0</v>
@@ -34158,10 +34158,10 @@
         <v>0.001582</v>
       </c>
       <c r="Y296" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z296" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA296" s="3" t="n">
         <v>1622</v>
@@ -35258,7 +35258,7 @@
         <v>0.001379</v>
       </c>
       <c r="Y307" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z307" s="3" t="n">
         <v>0</v>
@@ -35558,7 +35558,7 @@
         <v>0.00142</v>
       </c>
       <c r="Y310" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z310" s="3" t="n">
         <v>0</v>
@@ -36058,10 +36058,10 @@
         <v>0.001896</v>
       </c>
       <c r="Y315" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z315" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA315" s="3" t="n">
         <v>1537</v>
@@ -36361,7 +36361,7 @@
         <v>0</v>
       </c>
       <c r="Z318" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA318" s="3" t="n">
         <v>800</v>
@@ -36858,10 +36858,10 @@
         <v>0.001535</v>
       </c>
       <c r="Y323" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z323" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA323" s="3" t="n">
         <v>2054</v>
@@ -37258,7 +37258,7 @@
         <v>0.001423</v>
       </c>
       <c r="Y327" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z327" s="3" t="n">
         <v>0</v>
@@ -37558,10 +37558,10 @@
         <v>0.001302</v>
       </c>
       <c r="Y330" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z330" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA330" s="3" t="n">
         <v>849</v>
@@ -38558,10 +38558,10 @@
         <v>0.001476</v>
       </c>
       <c r="Y340" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z340" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA340" s="3" t="n">
         <v>556</v>
@@ -39258,10 +39258,10 @@
         <v>0.001345</v>
       </c>
       <c r="Y347" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z347" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA347" s="3" t="n">
         <v>1161</v>
@@ -39361,7 +39361,7 @@
         <v>0</v>
       </c>
       <c r="Z348" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA348" s="3" t="n">
         <v>1209</v>
@@ -39861,7 +39861,7 @@
         <v>-0</v>
       </c>
       <c r="Z353" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA353" s="3" t="n">
         <v>887</v>
@@ -39958,10 +39958,10 @@
         <v>0.001581</v>
       </c>
       <c r="Y354" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z354" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA354" s="3" t="n">
         <v>1125</v>
@@ -40958,10 +40958,10 @@
         <v>0.001262</v>
       </c>
       <c r="Y364" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z364" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA364" s="3" t="n">
         <v>708</v>
@@ -41661,7 +41661,7 @@
         <v>0</v>
       </c>
       <c r="Z371" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA371" s="3" t="n">
         <v>372</v>
@@ -42058,10 +42058,10 @@
         <v>0.000982</v>
       </c>
       <c r="Y375" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z375" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA375" s="3" t="n">
         <v>1642</v>
@@ -42358,7 +42358,7 @@
         <v>0.001213</v>
       </c>
       <c r="Y378" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z378" s="3" t="n">
         <v>-0</v>
@@ -42558,7 +42558,7 @@
         <v>0.00096</v>
       </c>
       <c r="Y380" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z380" s="3" t="n">
         <v>0</v>
@@ -43961,7 +43961,7 @@
         <v>0</v>
       </c>
       <c r="Z394" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA394" s="3" t="n">
         <v>428</v>
@@ -44058,10 +44058,10 @@
         <v>0.00096</v>
       </c>
       <c r="Y395" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z395" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA395" s="3" t="n">
         <v>648</v>
@@ -44158,10 +44158,10 @@
         <v>0.0009810000000000001</v>
       </c>
       <c r="Y396" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z396" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA396" s="3" t="n">
         <v>562</v>
@@ -44461,7 +44461,7 @@
         <v>0</v>
       </c>
       <c r="Z399" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA399" s="3" t="n">
         <v>506</v>
@@ -44558,10 +44558,10 @@
         <v>0.000806</v>
       </c>
       <c r="Y400" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z400" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA400" s="3" t="n">
         <v>643</v>
@@ -44740,10 +44740,10 @@
         <v>0.58377</v>
       </c>
       <c r="Y403" s="3" t="n">
-        <v>0.151043</v>
+        <v>0.108655</v>
       </c>
       <c r="Z403" s="3" t="n">
-        <v>0.158309</v>
+        <v>0.13215</v>
       </c>
       <c r="AA403" s="3" t="n">
         <v>0.6093150000000001</v>
@@ -44862,10 +44862,10 @@
         <v>0.810408</v>
       </c>
       <c r="Y407" s="3" t="n">
-        <v>-0.077877</v>
+        <v>-0.104138</v>
       </c>
       <c r="Z407" s="3" t="n">
-        <v>-0.088089</v>
+        <v>-0.090526</v>
       </c>
       <c r="AC407" s="3" t="n">
         <v>0.830507</v>
@@ -44881,10 +44881,10 @@
         <v>0.624937</v>
       </c>
       <c r="Y408" s="3" t="n">
-        <v>-0.050627</v>
+        <v>-0.070451</v>
       </c>
       <c r="Z408" s="3" t="n">
-        <v>-0.057168</v>
+        <v>-0.060777</v>
       </c>
       <c r="AC408" s="3" t="n">
         <v>0.646591</v>
@@ -45183,10 +45183,10 @@
         <v>0.467527</v>
       </c>
       <c r="D8" t="n">
-        <v>0.151043</v>
+        <v>0.108655</v>
       </c>
       <c r="E8" t="n">
-        <v>0.09948899999999999</v>
+        <v>0.067755</v>
       </c>
       <c r="F8" t="n">
         <v/>
@@ -45243,10 +45243,10 @@
         <v>0.649212</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.077877</v>
+        <v>-0.104138</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.050627</v>
+        <v>-0.070451</v>
       </c>
       <c r="F10" t="n">
         <v/>
@@ -45273,10 +45273,10 @@
         <v>0.467574</v>
       </c>
       <c r="D11" t="n">
-        <v>0.158309</v>
+        <v>0.13215</v>
       </c>
       <c r="E11" t="n">
-        <v>0.105179</v>
+        <v>0.087006</v>
       </c>
       <c r="F11" t="n">
         <v/>
@@ -45333,10 +45333,10 @@
         <v>0.649384</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.088089</v>
+        <v>-0.090526</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.057168</v>
+        <v>-0.060777</v>
       </c>
       <c r="F13" t="n">
         <v/>

</xml_diff>

<commit_message>
feat(epirank): replace enterovirus with norovirus (nv.xlsx) in both Germany variants
- EpiRank_GUI.py (原/改/reverse): KEY_EV_AVERAGE_CASES -> KEY_NV_TOTAL_CASES, ev.xlsx -> nv.xlsx, ev_cases/nv_cases fields, int case counts
- add nv.xlsx case tables to 原_Germany and 改_Germany
- add 原始数据/norovirus_germany_county_2015_2020_raw.csv and 疾病数据说明.md
- regenerate ERA_result_*.json/xlsx for 原 (daytime 0.5, 110 loops) and 改 (seqday/reverse, 105 loops)
</commit_message>
<xml_diff>
--- a/EpiRank_原_Germany/ERA_result_d_0.95_daytime_0.5_loops_110.xlsx
+++ b/EpiRank_原_Germany/ERA_result_d_0.95_daytime_0.5_loops_110.xlsx
@@ -575,7 +575,7 @@
       </c>
       <c r="AB1" s="2" t="inlineStr">
         <is>
-          <t>ev cases</t>
+          <t>nv cases</t>
         </is>
       </c>
       <c r="AC1" s="2" t="inlineStr">
@@ -723,7 +723,7 @@
         <v>35664</v>
       </c>
       <c r="AB2" s="3" t="n">
-        <v>0</v>
+        <v>29116</v>
       </c>
       <c r="AC2" s="3" t="n">
         <v>1477017</v>
@@ -868,7 +868,7 @@
         <v>34035</v>
       </c>
       <c r="AB3" s="3" t="n">
-        <v>0</v>
+        <v>7880</v>
       </c>
       <c r="AC3" s="3" t="n">
         <v>736525</v>
@@ -1013,7 +1013,7 @@
         <v>27918</v>
       </c>
       <c r="AB4" s="3" t="n">
-        <v>0</v>
+        <v>11726</v>
       </c>
       <c r="AC4" s="3" t="n">
         <v>828151</v>
@@ -1158,7 +1158,7 @@
         <v>8482</v>
       </c>
       <c r="AB5" s="3" t="n">
-        <v>0</v>
+        <v>4477</v>
       </c>
       <c r="AC5" s="3" t="n">
         <v>549016</v>
@@ -1303,7 +1303,7 @@
         <v>7677</v>
       </c>
       <c r="AB6" s="3" t="n">
-        <v>0</v>
+        <v>1465</v>
       </c>
       <c r="AC6" s="3" t="n">
         <v>263686</v>
@@ -1435,7 +1435,7 @@
         <v>0.01118</v>
       </c>
       <c r="Y7" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z7" s="3" t="n">
         <v>-0</v>
@@ -1444,7 +1444,7 @@
         <v>6805</v>
       </c>
       <c r="AB7" s="3" t="n">
-        <v>0</v>
+        <v>3551</v>
       </c>
       <c r="AC7" s="3" t="n">
         <v>341931</v>
@@ -1585,7 +1585,7 @@
         <v>8532</v>
       </c>
       <c r="AB8" s="3" t="n">
-        <v>0</v>
+        <v>4129</v>
       </c>
       <c r="AC8" s="3" t="n">
         <v>522328</v>
@@ -1726,7 +1726,7 @@
         <v>1462</v>
       </c>
       <c r="AB9" s="3" t="n">
-        <v>0</v>
+        <v>2601</v>
       </c>
       <c r="AC9" s="3" t="n">
         <v>255121</v>
@@ -1867,7 +1867,7 @@
         <v>25337</v>
       </c>
       <c r="AB10" s="3" t="n">
-        <v>67</v>
+        <v>4683</v>
       </c>
       <c r="AC10" s="3" t="n">
         <v>293090</v>
@@ -2012,7 +2012,7 @@
         <v>7136</v>
       </c>
       <c r="AB11" s="3" t="n">
-        <v>0</v>
+        <v>2405</v>
       </c>
       <c r="AC11" s="3" t="n">
         <v>254011</v>
@@ -2148,16 +2148,16 @@
         <v>0.007346</v>
       </c>
       <c r="Y12" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z12" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA12" s="3" t="n">
         <v>6490</v>
       </c>
       <c r="AB12" s="3" t="n">
-        <v>0</v>
+        <v>2130</v>
       </c>
       <c r="AC12" s="3" t="n">
         <v>258750</v>
@@ -2302,7 +2302,7 @@
         <v>1620</v>
       </c>
       <c r="AB13" s="3" t="n">
-        <v>0</v>
+        <v>2624</v>
       </c>
       <c r="AC13" s="3" t="n">
         <v>157291</v>
@@ -2437,7 +2437,7 @@
         <v>13685</v>
       </c>
       <c r="AB14" s="3" t="n">
-        <v>38</v>
+        <v>4154</v>
       </c>
       <c r="AC14" s="3" t="n">
         <v>289842</v>
@@ -2567,7 +2567,7 @@
         <v>4465</v>
       </c>
       <c r="AB15" s="3" t="n">
-        <v>0</v>
+        <v>2941</v>
       </c>
       <c r="AC15" s="3" t="n">
         <v>284086</v>
@@ -2688,16 +2688,16 @@
         <v>0.005427</v>
       </c>
       <c r="Y16" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z16" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA16" s="3" t="n">
         <v>1918</v>
       </c>
       <c r="AB16" s="3" t="n">
-        <v>0</v>
+        <v>2683</v>
       </c>
       <c r="AC16" s="3" t="n">
         <v>235685</v>
@@ -2827,7 +2827,7 @@
         <v>4952</v>
       </c>
       <c r="AB17" s="3" t="n">
-        <v>0</v>
+        <v>3407</v>
       </c>
       <c r="AC17" s="3" t="n">
         <v>269074</v>
@@ -2947,7 +2947,7 @@
         <v>2380</v>
       </c>
       <c r="AB18" s="3" t="n">
-        <v>0</v>
+        <v>2684</v>
       </c>
       <c r="AC18" s="3" t="n">
         <v>267206</v>
@@ -3067,7 +3067,7 @@
         <v>6813</v>
       </c>
       <c r="AB19" s="3" t="n">
-        <v>0</v>
+        <v>2250</v>
       </c>
       <c r="AC19" s="3" t="n">
         <v>238986</v>
@@ -3178,16 +3178,16 @@
         <v>0.004953</v>
       </c>
       <c r="Y20" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z20" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA20" s="3" t="n">
         <v>4207</v>
       </c>
       <c r="AB20" s="3" t="n">
-        <v>0</v>
+        <v>1959</v>
       </c>
       <c r="AC20" s="3" t="n">
         <v>247527</v>
@@ -3307,7 +3307,7 @@
         <v>4867</v>
       </c>
       <c r="AB21" s="3" t="n">
-        <v>0</v>
+        <v>4657</v>
       </c>
       <c r="AC21" s="3" t="n">
         <v>211676</v>
@@ -3427,7 +3427,7 @@
         <v>4123</v>
       </c>
       <c r="AB22" s="3" t="n">
-        <v>0</v>
+        <v>1742</v>
       </c>
       <c r="AC22" s="3" t="n">
         <v>214509</v>
@@ -3547,7 +3547,7 @@
         <v>3797</v>
       </c>
       <c r="AB23" s="3" t="n">
-        <v>0</v>
+        <v>3769</v>
       </c>
       <c r="AC23" s="3" t="n">
         <v>83977</v>
@@ -3667,7 +3667,7 @@
         <v>2908</v>
       </c>
       <c r="AB24" s="3" t="n">
-        <v>0</v>
+        <v>2603</v>
       </c>
       <c r="AC24" s="3" t="n">
         <v>159960</v>
@@ -3778,16 +3778,16 @@
         <v>0.004167</v>
       </c>
       <c r="Y25" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z25" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA25" s="3" t="n">
         <v>3606</v>
       </c>
       <c r="AB25" s="3" t="n">
-        <v>0</v>
+        <v>2623</v>
       </c>
       <c r="AC25" s="3" t="n">
         <v>215076</v>
@@ -3907,7 +3907,7 @@
         <v>3006</v>
       </c>
       <c r="AB26" s="3" t="n">
-        <v>0</v>
+        <v>2215</v>
       </c>
       <c r="AC26" s="3" t="n">
         <v>139375</v>
@@ -4027,7 +4027,7 @@
         <v>1432</v>
       </c>
       <c r="AB27" s="3" t="n">
-        <v>0</v>
+        <v>1468</v>
       </c>
       <c r="AC27" s="3" t="n">
         <v>147675</v>
@@ -4138,16 +4138,16 @@
         <v>0.004224</v>
       </c>
       <c r="Y28" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z28" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA28" s="3" t="n">
         <v>3369</v>
       </c>
       <c r="AB28" s="3" t="n">
-        <v>0</v>
+        <v>3996</v>
       </c>
       <c r="AC28" s="3" t="n">
         <v>254023</v>
@@ -4258,16 +4258,16 @@
         <v>0.003699</v>
       </c>
       <c r="Y29" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z29" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA29" s="3" t="n">
         <v>2262</v>
       </c>
       <c r="AB29" s="3" t="n">
-        <v>0</v>
+        <v>3157</v>
       </c>
       <c r="AC29" s="3" t="n">
         <v>262194</v>
@@ -4387,7 +4387,7 @@
         <v>2551</v>
       </c>
       <c r="AB30" s="3" t="n">
-        <v>0</v>
+        <v>1131</v>
       </c>
       <c r="AC30" s="3" t="n">
         <v>133058</v>
@@ -4507,7 +4507,7 @@
         <v>5165</v>
       </c>
       <c r="AB31" s="3" t="n">
-        <v>0</v>
+        <v>2601</v>
       </c>
       <c r="AC31" s="3" t="n">
         <v>218319</v>
@@ -4627,7 +4627,7 @@
         <v>7852</v>
       </c>
       <c r="AB32" s="3" t="n">
-        <v>2</v>
+        <v>4089</v>
       </c>
       <c r="AC32" s="3" t="n">
         <v>151232</v>
@@ -4747,7 +4747,7 @@
         <v>3059</v>
       </c>
       <c r="AB33" s="3" t="n">
-        <v>0</v>
+        <v>1465</v>
       </c>
       <c r="AC33" s="3" t="n">
         <v>132271</v>
@@ -4858,16 +4858,16 @@
         <v>0.004134</v>
       </c>
       <c r="Y34" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z34" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA34" s="3" t="n">
         <v>3860</v>
       </c>
       <c r="AB34" s="3" t="n">
-        <v>0</v>
+        <v>1551</v>
       </c>
       <c r="AC34" s="3" t="n">
         <v>200571</v>
@@ -4978,16 +4978,16 @@
         <v>0.004087</v>
       </c>
       <c r="Y35" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z35" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA35" s="3" t="n">
         <v>2538</v>
       </c>
       <c r="AB35" s="3" t="n">
-        <v>0</v>
+        <v>2703</v>
       </c>
       <c r="AC35" s="3" t="n">
         <v>167225</v>
@@ -5107,7 +5107,7 @@
         <v>11679</v>
       </c>
       <c r="AB36" s="3" t="n">
-        <v>0</v>
+        <v>1646</v>
       </c>
       <c r="AC36" s="3" t="n">
         <v>170202</v>
@@ -5218,16 +5218,16 @@
         <v>0.003682</v>
       </c>
       <c r="Y37" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z37" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA37" s="3" t="n">
         <v>2678</v>
       </c>
       <c r="AB37" s="3" t="n">
-        <v>0</v>
+        <v>1135</v>
       </c>
       <c r="AC37" s="3" t="n">
         <v>154363</v>
@@ -5341,13 +5341,13 @@
         <v>0</v>
       </c>
       <c r="Z38" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA38" s="3" t="n">
         <v>7680</v>
       </c>
       <c r="AB38" s="3" t="n">
-        <v>0</v>
+        <v>1816</v>
       </c>
       <c r="AC38" s="3" t="n">
         <v>107335</v>
@@ -5467,7 +5467,7 @@
         <v>1117</v>
       </c>
       <c r="AB39" s="3" t="n">
-        <v>0</v>
+        <v>1214</v>
       </c>
       <c r="AC39" s="3" t="n">
         <v>113148</v>
@@ -5578,7 +5578,7 @@
         <v>0.003994</v>
       </c>
       <c r="Y40" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z40" s="3" t="n">
         <v>0</v>
@@ -5587,7 +5587,7 @@
         <v>2893</v>
       </c>
       <c r="AB40" s="3" t="n">
-        <v>0</v>
+        <v>1704</v>
       </c>
       <c r="AC40" s="3" t="n">
         <v>169197</v>
@@ -5707,7 +5707,7 @@
         <v>5600</v>
       </c>
       <c r="AB41" s="3" t="n">
-        <v>0</v>
+        <v>4264</v>
       </c>
       <c r="AC41" s="3" t="n">
         <v>93342</v>
@@ -5827,7 +5827,7 @@
         <v>3417</v>
       </c>
       <c r="AB42" s="3" t="n">
-        <v>0</v>
+        <v>1002</v>
       </c>
       <c r="AC42" s="3" t="n">
         <v>186667</v>
@@ -5947,7 +5947,7 @@
         <v>2060</v>
       </c>
       <c r="AB43" s="3" t="n">
-        <v>0</v>
+        <v>1436</v>
       </c>
       <c r="AC43" s="3" t="n">
         <v>172067</v>
@@ -6067,7 +6067,7 @@
         <v>2752</v>
       </c>
       <c r="AB44" s="3" t="n">
-        <v>0</v>
+        <v>1378</v>
       </c>
       <c r="AC44" s="3" t="n">
         <v>150423</v>
@@ -6187,7 +6187,7 @@
         <v>3379</v>
       </c>
       <c r="AB45" s="3" t="n">
-        <v>0</v>
+        <v>1949</v>
       </c>
       <c r="AC45" s="3" t="n">
         <v>198424</v>
@@ -6307,7 +6307,7 @@
         <v>1989</v>
       </c>
       <c r="AB46" s="3" t="n">
-        <v>0</v>
+        <v>2578</v>
       </c>
       <c r="AC46" s="3" t="n">
         <v>136372</v>
@@ -6427,7 +6427,7 @@
         <v>10878</v>
       </c>
       <c r="AB47" s="3" t="n">
-        <v>3</v>
+        <v>4308</v>
       </c>
       <c r="AC47" s="3" t="n">
         <v>167986</v>
@@ -6547,7 +6547,7 @@
         <v>548</v>
       </c>
       <c r="AB48" s="3" t="n">
-        <v>0</v>
+        <v>905</v>
       </c>
       <c r="AC48" s="3" t="n">
         <v>90630</v>
@@ -6658,16 +6658,16 @@
         <v>0.003683</v>
       </c>
       <c r="Y49" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z49" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA49" s="3" t="n">
         <v>2526</v>
       </c>
       <c r="AB49" s="3" t="n">
-        <v>0</v>
+        <v>3903</v>
       </c>
       <c r="AC49" s="3" t="n">
         <v>238412</v>
@@ -6787,7 +6787,7 @@
         <v>2064</v>
       </c>
       <c r="AB50" s="3" t="n">
-        <v>0</v>
+        <v>2076</v>
       </c>
       <c r="AC50" s="3" t="n">
         <v>167127</v>
@@ -6907,7 +6907,7 @@
         <v>5461</v>
       </c>
       <c r="AB51" s="3" t="n">
-        <v>2</v>
+        <v>2706</v>
       </c>
       <c r="AC51" s="3" t="n">
         <v>113002</v>
@@ -7027,7 +7027,7 @@
         <v>1472</v>
       </c>
       <c r="AB52" s="3" t="n">
-        <v>0</v>
+        <v>897</v>
       </c>
       <c r="AC52" s="3" t="n">
         <v>126408</v>
@@ -7147,7 +7147,7 @@
         <v>3344</v>
       </c>
       <c r="AB53" s="3" t="n">
-        <v>0</v>
+        <v>1851</v>
       </c>
       <c r="AC53" s="3" t="n">
         <v>138200</v>
@@ -7261,13 +7261,13 @@
         <v>0</v>
       </c>
       <c r="Z54" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA54" s="3" t="n">
         <v>930</v>
       </c>
       <c r="AB54" s="3" t="n">
-        <v>0</v>
+        <v>1093</v>
       </c>
       <c r="AC54" s="3" t="n">
         <v>134090</v>
@@ -7387,7 +7387,7 @@
         <v>2152</v>
       </c>
       <c r="AB55" s="3" t="n">
-        <v>0</v>
+        <v>2187</v>
       </c>
       <c r="AC55" s="3" t="n">
         <v>204631</v>
@@ -7501,13 +7501,13 @@
         <v>0</v>
       </c>
       <c r="Z56" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA56" s="3" t="n">
         <v>1130</v>
       </c>
       <c r="AB56" s="3" t="n">
-        <v>0</v>
+        <v>1585</v>
       </c>
       <c r="AC56" s="3" t="n">
         <v>104492</v>
@@ -7621,13 +7621,13 @@
         <v>-0</v>
       </c>
       <c r="Z57" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA57" s="3" t="n">
         <v>1293</v>
       </c>
       <c r="AB57" s="3" t="n">
-        <v>0</v>
+        <v>1252</v>
       </c>
       <c r="AC57" s="3" t="n">
         <v>128863</v>
@@ -7747,7 +7747,7 @@
         <v>5618</v>
       </c>
       <c r="AB58" s="3" t="n">
-        <v>0</v>
+        <v>671</v>
       </c>
       <c r="AC58" s="3" t="n">
         <v>107984</v>
@@ -7867,7 +7867,7 @@
         <v>4129</v>
       </c>
       <c r="AB59" s="3" t="n">
-        <v>0</v>
+        <v>1292</v>
       </c>
       <c r="AC59" s="3" t="n">
         <v>194254</v>
@@ -7987,7 +7987,7 @@
         <v>2142</v>
       </c>
       <c r="AB60" s="3" t="n">
-        <v>0</v>
+        <v>1094</v>
       </c>
       <c r="AC60" s="3" t="n">
         <v>133690</v>
@@ -8107,7 +8107,7 @@
         <v>4171</v>
       </c>
       <c r="AB61" s="3" t="n">
-        <v>0</v>
+        <v>2128</v>
       </c>
       <c r="AC61" s="3" t="n">
         <v>105697</v>
@@ -8227,7 +8227,7 @@
         <v>2122</v>
       </c>
       <c r="AB62" s="3" t="n">
-        <v>0</v>
+        <v>2648</v>
       </c>
       <c r="AC62" s="3" t="n">
         <v>156360</v>
@@ -8338,7 +8338,7 @@
         <v>0.003143</v>
       </c>
       <c r="Y63" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z63" s="3" t="n">
         <v>-0</v>
@@ -8347,7 +8347,7 @@
         <v>2303</v>
       </c>
       <c r="AB63" s="3" t="n">
-        <v>0</v>
+        <v>2241</v>
       </c>
       <c r="AC63" s="3" t="n">
         <v>236874</v>
@@ -8467,7 +8467,7 @@
         <v>3819</v>
       </c>
       <c r="AB64" s="3" t="n">
-        <v>0</v>
+        <v>486</v>
       </c>
       <c r="AC64" s="3" t="n">
         <v>78578</v>
@@ -8587,7 +8587,7 @@
         <v>2463</v>
       </c>
       <c r="AB65" s="3" t="n">
-        <v>0</v>
+        <v>1263</v>
       </c>
       <c r="AC65" s="3" t="n">
         <v>115651</v>
@@ -8707,7 +8707,7 @@
         <v>2443</v>
       </c>
       <c r="AB66" s="3" t="n">
-        <v>0</v>
+        <v>2283</v>
       </c>
       <c r="AC66" s="3" t="n">
         <v>201013</v>
@@ -8827,7 +8827,7 @@
         <v>2734</v>
       </c>
       <c r="AB67" s="3" t="n">
-        <v>0</v>
+        <v>1935</v>
       </c>
       <c r="AC67" s="3" t="n">
         <v>185793</v>
@@ -8947,7 +8947,7 @@
         <v>2101</v>
       </c>
       <c r="AB68" s="3" t="n">
-        <v>0</v>
+        <v>1670</v>
       </c>
       <c r="AC68" s="3" t="n">
         <v>138620</v>
@@ -9067,7 +9067,7 @@
         <v>9844</v>
       </c>
       <c r="AB69" s="3" t="n">
-        <v>6</v>
+        <v>3710</v>
       </c>
       <c r="AC69" s="3" t="n">
         <v>160814</v>
@@ -9187,7 +9187,7 @@
         <v>11662</v>
       </c>
       <c r="AB70" s="3" t="n">
-        <v>0</v>
+        <v>3951</v>
       </c>
       <c r="AC70" s="3" t="n">
         <v>145072</v>
@@ -9307,7 +9307,7 @@
         <v>1701</v>
       </c>
       <c r="AB71" s="3" t="n">
-        <v>0</v>
+        <v>1694</v>
       </c>
       <c r="AC71" s="3" t="n">
         <v>179203</v>
@@ -9427,7 +9427,7 @@
         <v>3557</v>
       </c>
       <c r="AB72" s="3" t="n">
-        <v>0</v>
+        <v>1502</v>
       </c>
       <c r="AC72" s="3" t="n">
         <v>134853</v>
@@ -9547,7 +9547,7 @@
         <v>11227</v>
       </c>
       <c r="AB73" s="3" t="n">
-        <v>0</v>
+        <v>4580</v>
       </c>
       <c r="AC73" s="3" t="n">
         <v>113929</v>
@@ -9667,7 +9667,7 @@
         <v>2524</v>
       </c>
       <c r="AB74" s="3" t="n">
-        <v>0</v>
+        <v>1620</v>
       </c>
       <c r="AC74" s="3" t="n">
         <v>143663</v>
@@ -9778,16 +9778,16 @@
         <v>0.003381</v>
       </c>
       <c r="Y75" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z75" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA75" s="3" t="n">
         <v>1306</v>
       </c>
       <c r="AB75" s="3" t="n">
-        <v>0</v>
+        <v>1738</v>
       </c>
       <c r="AC75" s="3" t="n">
         <v>175579</v>
@@ -9907,7 +9907,7 @@
         <v>1868</v>
       </c>
       <c r="AB76" s="3" t="n">
-        <v>0</v>
+        <v>1859</v>
       </c>
       <c r="AC76" s="3" t="n">
         <v>124289</v>
@@ -10027,7 +10027,7 @@
         <v>2678</v>
       </c>
       <c r="AB77" s="3" t="n">
-        <v>0</v>
+        <v>2266</v>
       </c>
       <c r="AC77" s="3" t="n">
         <v>140016</v>
@@ -10147,7 +10147,7 @@
         <v>2935</v>
       </c>
       <c r="AB78" s="3" t="n">
-        <v>0</v>
+        <v>569</v>
       </c>
       <c r="AC78" s="3" t="n">
         <v>86794</v>
@@ -10267,7 +10267,7 @@
         <v>3171</v>
       </c>
       <c r="AB79" s="3" t="n">
-        <v>0</v>
+        <v>2624</v>
       </c>
       <c r="AC79" s="3" t="n">
         <v>198885</v>
@@ -10387,7 +10387,7 @@
         <v>1537</v>
       </c>
       <c r="AB80" s="3" t="n">
-        <v>0</v>
+        <v>970</v>
       </c>
       <c r="AC80" s="3" t="n">
         <v>101231</v>
@@ -10501,13 +10501,13 @@
         <v>0</v>
       </c>
       <c r="Z81" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA81" s="3" t="n">
         <v>871</v>
       </c>
       <c r="AB81" s="3" t="n">
-        <v>0</v>
+        <v>1073</v>
       </c>
       <c r="AC81" s="3" t="n">
         <v>134524</v>
@@ -10627,7 +10627,7 @@
         <v>1694</v>
       </c>
       <c r="AB82" s="3" t="n">
-        <v>0</v>
+        <v>2091</v>
       </c>
       <c r="AC82" s="3" t="n">
         <v>133621</v>
@@ -10747,7 +10747,7 @@
         <v>3194</v>
       </c>
       <c r="AB83" s="3" t="n">
-        <v>0</v>
+        <v>2985</v>
       </c>
       <c r="AC83" s="3" t="n">
         <v>149832</v>
@@ -10867,7 +10867,7 @@
         <v>2602</v>
       </c>
       <c r="AB84" s="3" t="n">
-        <v>0</v>
+        <v>2392</v>
       </c>
       <c r="AC84" s="3" t="n">
         <v>173030</v>
@@ -10987,7 +10987,7 @@
         <v>2843</v>
       </c>
       <c r="AB85" s="3" t="n">
-        <v>0</v>
+        <v>1286</v>
       </c>
       <c r="AC85" s="3" t="n">
         <v>94308</v>
@@ -11107,7 +11107,7 @@
         <v>671</v>
       </c>
       <c r="AB86" s="3" t="n">
-        <v>0</v>
+        <v>544</v>
       </c>
       <c r="AC86" s="3" t="n">
         <v>81048</v>
@@ -11227,7 +11227,7 @@
         <v>1414</v>
       </c>
       <c r="AB87" s="3" t="n">
-        <v>0</v>
+        <v>842</v>
       </c>
       <c r="AC87" s="3" t="n">
         <v>81733</v>
@@ -11347,7 +11347,7 @@
         <v>1943</v>
       </c>
       <c r="AB88" s="3" t="n">
-        <v>0</v>
+        <v>1094</v>
       </c>
       <c r="AC88" s="3" t="n">
         <v>98098</v>
@@ -11467,7 +11467,7 @@
         <v>1151</v>
       </c>
       <c r="AB89" s="3" t="n">
-        <v>0</v>
+        <v>1035</v>
       </c>
       <c r="AC89" s="3" t="n">
         <v>70779</v>
@@ -11587,7 +11587,7 @@
         <v>5293</v>
       </c>
       <c r="AB90" s="3" t="n">
-        <v>0</v>
+        <v>1799</v>
       </c>
       <c r="AC90" s="3" t="n">
         <v>82617</v>
@@ -11707,7 +11707,7 @@
         <v>2304</v>
       </c>
       <c r="AB91" s="3" t="n">
-        <v>0</v>
+        <v>2524</v>
       </c>
       <c r="AC91" s="3" t="n">
         <v>98857</v>
@@ -11827,7 +11827,7 @@
         <v>765</v>
       </c>
       <c r="AB92" s="3" t="n">
-        <v>0</v>
+        <v>870</v>
       </c>
       <c r="AC92" s="3" t="n">
         <v>122290</v>
@@ -11947,7 +11947,7 @@
         <v>3690</v>
       </c>
       <c r="AB93" s="3" t="n">
-        <v>0</v>
+        <v>1638</v>
       </c>
       <c r="AC93" s="3" t="n">
         <v>150752</v>
@@ -12067,7 +12067,7 @@
         <v>1472</v>
       </c>
       <c r="AB94" s="3" t="n">
-        <v>0</v>
+        <v>497</v>
       </c>
       <c r="AC94" s="3" t="n">
         <v>103066</v>
@@ -12187,7 +12187,7 @@
         <v>7421</v>
       </c>
       <c r="AB95" s="3" t="n">
-        <v>0</v>
+        <v>2798</v>
       </c>
       <c r="AC95" s="3" t="n">
         <v>113041</v>
@@ -12307,7 +12307,7 @@
         <v>3818</v>
       </c>
       <c r="AB96" s="3" t="n">
-        <v>0</v>
+        <v>2938</v>
       </c>
       <c r="AC96" s="3" t="n">
         <v>199738</v>
@@ -12427,7 +12427,7 @@
         <v>3061</v>
       </c>
       <c r="AB97" s="3" t="n">
-        <v>0</v>
+        <v>3431</v>
       </c>
       <c r="AC97" s="3" t="n">
         <v>95398</v>
@@ -12547,7 +12547,7 @@
         <v>5645</v>
       </c>
       <c r="AB98" s="3" t="n">
-        <v>0</v>
+        <v>1174</v>
       </c>
       <c r="AC98" s="3" t="n">
         <v>81009</v>
@@ -12667,7 +12667,7 @@
         <v>2203</v>
       </c>
       <c r="AB99" s="3" t="n">
-        <v>0</v>
+        <v>941</v>
       </c>
       <c r="AC99" s="3" t="n">
         <v>101511</v>
@@ -12787,7 +12787,7 @@
         <v>12443</v>
       </c>
       <c r="AB100" s="3" t="n">
-        <v>11</v>
+        <v>3476</v>
       </c>
       <c r="AC100" s="3" t="n">
         <v>134228</v>
@@ -12901,13 +12901,13 @@
         <v>0</v>
       </c>
       <c r="Z101" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA101" s="3" t="n">
         <v>1745</v>
       </c>
       <c r="AB101" s="3" t="n">
-        <v>0</v>
+        <v>710</v>
       </c>
       <c r="AC101" s="3" t="n">
         <v>114450</v>
@@ -13027,7 +13027,7 @@
         <v>3835</v>
       </c>
       <c r="AB102" s="3" t="n">
-        <v>0</v>
+        <v>730</v>
       </c>
       <c r="AC102" s="3" t="n">
         <v>108098</v>
@@ -13147,7 +13147,7 @@
         <v>1288</v>
       </c>
       <c r="AB103" s="3" t="n">
-        <v>0</v>
+        <v>454</v>
       </c>
       <c r="AC103" s="3" t="n">
         <v>70204</v>
@@ -13267,7 +13267,7 @@
         <v>8108</v>
       </c>
       <c r="AB104" s="3" t="n">
-        <v>0</v>
+        <v>3997</v>
       </c>
       <c r="AC104" s="3" t="n">
         <v>98352</v>
@@ -13378,16 +13378,16 @@
         <v>0.002646</v>
       </c>
       <c r="Y105" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z105" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA105" s="3" t="n">
         <v>4116</v>
       </c>
       <c r="AB105" s="3" t="n">
-        <v>0</v>
+        <v>1041</v>
       </c>
       <c r="AC105" s="3" t="n">
         <v>119264</v>
@@ -13498,7 +13498,7 @@
         <v>0.002503</v>
       </c>
       <c r="Y106" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z106" s="3" t="n">
         <v>0</v>
@@ -13507,7 +13507,7 @@
         <v>1871</v>
       </c>
       <c r="AB106" s="3" t="n">
-        <v>0</v>
+        <v>1654</v>
       </c>
       <c r="AC106" s="3" t="n">
         <v>102080</v>
@@ -13627,7 +13627,7 @@
         <v>1575</v>
       </c>
       <c r="AB107" s="3" t="n">
-        <v>0</v>
+        <v>543</v>
       </c>
       <c r="AC107" s="3" t="n">
         <v>83461</v>
@@ -13747,7 +13747,7 @@
         <v>1724</v>
       </c>
       <c r="AB108" s="3" t="n">
-        <v>0</v>
+        <v>1146</v>
       </c>
       <c r="AC108" s="3" t="n">
         <v>125917</v>
@@ -13858,16 +13858,16 @@
         <v>0.002608</v>
       </c>
       <c r="Y109" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z109" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA109" s="3" t="n">
         <v>3508</v>
       </c>
       <c r="AB109" s="3" t="n">
-        <v>0</v>
+        <v>1384</v>
       </c>
       <c r="AC109" s="3" t="n">
         <v>116851</v>
@@ -13978,16 +13978,16 @@
         <v>0.002646</v>
       </c>
       <c r="Y110" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z110" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA110" s="3" t="n">
         <v>2711</v>
       </c>
       <c r="AB110" s="3" t="n">
-        <v>0</v>
+        <v>1760</v>
       </c>
       <c r="AC110" s="3" t="n">
         <v>99164</v>
@@ -14107,7 +14107,7 @@
         <v>4089</v>
       </c>
       <c r="AB111" s="3" t="n">
-        <v>0</v>
+        <v>841</v>
       </c>
       <c r="AC111" s="3" t="n">
         <v>88872</v>
@@ -14227,7 +14227,7 @@
         <v>969</v>
       </c>
       <c r="AB112" s="3" t="n">
-        <v>0</v>
+        <v>1423</v>
       </c>
       <c r="AC112" s="3" t="n">
         <v>130625</v>
@@ -14347,7 +14347,7 @@
         <v>1092</v>
       </c>
       <c r="AB113" s="3" t="n">
-        <v>0</v>
+        <v>677</v>
       </c>
       <c r="AC113" s="3" t="n">
         <v>70552</v>
@@ -14467,7 +14467,7 @@
         <v>1419</v>
       </c>
       <c r="AB114" s="3" t="n">
-        <v>0</v>
+        <v>1794</v>
       </c>
       <c r="AC114" s="3" t="n">
         <v>66996</v>
@@ -14587,7 +14587,7 @@
         <v>5482</v>
       </c>
       <c r="AB115" s="3" t="n">
-        <v>0</v>
+        <v>2095</v>
       </c>
       <c r="AC115" s="3" t="n">
         <v>130239</v>
@@ -14701,13 +14701,13 @@
         <v>0</v>
       </c>
       <c r="Z116" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA116" s="3" t="n">
         <v>2287</v>
       </c>
       <c r="AB116" s="3" t="n">
-        <v>0</v>
+        <v>1744</v>
       </c>
       <c r="AC116" s="3" t="n">
         <v>69784</v>
@@ -14827,7 +14827,7 @@
         <v>3242</v>
       </c>
       <c r="AB117" s="3" t="n">
-        <v>0</v>
+        <v>2055</v>
       </c>
       <c r="AC117" s="3" t="n">
         <v>54219</v>
@@ -14937,7 +14937,7 @@
         <v>3944</v>
       </c>
       <c r="AB118" s="3" t="n">
-        <v>0</v>
+        <v>2409</v>
       </c>
       <c r="AC118" s="3" t="n">
         <v>49283</v>
@@ -15047,7 +15047,7 @@
         <v>3031</v>
       </c>
       <c r="AB119" s="3" t="n">
-        <v>0</v>
+        <v>4360</v>
       </c>
       <c r="AC119" s="3" t="n">
         <v>99946</v>
@@ -15157,7 +15157,7 @@
         <v>1080</v>
       </c>
       <c r="AB120" s="3" t="n">
-        <v>0</v>
+        <v>1457</v>
       </c>
       <c r="AC120" s="3" t="n">
         <v>82227</v>
@@ -15267,7 +15267,7 @@
         <v>1123</v>
       </c>
       <c r="AB121" s="3" t="n">
-        <v>0</v>
+        <v>4072</v>
       </c>
       <c r="AC121" s="3" t="n">
         <v>121897</v>
@@ -15377,7 +15377,7 @@
         <v>3092</v>
       </c>
       <c r="AB122" s="3" t="n">
-        <v>0</v>
+        <v>370</v>
       </c>
       <c r="AC122" s="3" t="n">
         <v>71122</v>
@@ -15478,16 +15478,16 @@
         <v>0.002324</v>
       </c>
       <c r="Y123" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z123" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA123" s="3" t="n">
         <v>2532</v>
       </c>
       <c r="AB123" s="3" t="n">
-        <v>0</v>
+        <v>936</v>
       </c>
       <c r="AC123" s="3" t="n">
         <v>102505</v>
@@ -15591,13 +15591,13 @@
         <v>0</v>
       </c>
       <c r="Z124" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA124" s="3" t="n">
         <v>5101</v>
       </c>
       <c r="AB124" s="3" t="n">
-        <v>0</v>
+        <v>1026</v>
       </c>
       <c r="AC124" s="3" t="n">
         <v>62638</v>
@@ -15701,13 +15701,13 @@
         <v>-0</v>
       </c>
       <c r="Z125" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA125" s="3" t="n">
         <v>1517</v>
       </c>
       <c r="AB125" s="3" t="n">
-        <v>0</v>
+        <v>846</v>
       </c>
       <c r="AC125" s="3" t="n">
         <v>112891</v>
@@ -15817,7 +15817,7 @@
         <v>1796</v>
       </c>
       <c r="AB126" s="3" t="n">
-        <v>0</v>
+        <v>969</v>
       </c>
       <c r="AC126" s="3" t="n">
         <v>96559</v>
@@ -15927,7 +15927,7 @@
         <v>1027</v>
       </c>
       <c r="AB127" s="3" t="n">
-        <v>0</v>
+        <v>1803</v>
       </c>
       <c r="AC127" s="3" t="n">
         <v>58587</v>
@@ -16037,7 +16037,7 @@
         <v>2260</v>
       </c>
       <c r="AB128" s="3" t="n">
-        <v>0</v>
+        <v>517</v>
       </c>
       <c r="AC128" s="3" t="n">
         <v>74485</v>
@@ -16147,7 +16147,7 @@
         <v>2832</v>
       </c>
       <c r="AB129" s="3" t="n">
-        <v>0</v>
+        <v>4744</v>
       </c>
       <c r="AC129" s="3" t="n">
         <v>102793</v>
@@ -16257,7 +16257,7 @@
         <v>2127</v>
       </c>
       <c r="AB130" s="3" t="n">
-        <v>0</v>
+        <v>2482</v>
       </c>
       <c r="AC130" s="3" t="n">
         <v>94208</v>
@@ -16367,7 +16367,7 @@
         <v>2916</v>
       </c>
       <c r="AB131" s="3" t="n">
-        <v>0</v>
+        <v>1196</v>
       </c>
       <c r="AC131" s="3" t="n">
         <v>81086</v>
@@ -16477,7 +16477,7 @@
         <v>609</v>
       </c>
       <c r="AB132" s="3" t="n">
-        <v>0</v>
+        <v>2369</v>
       </c>
       <c r="AC132" s="3" t="n">
         <v>49759</v>
@@ -16587,7 +16587,7 @@
         <v>1776</v>
       </c>
       <c r="AB133" s="3" t="n">
-        <v>0</v>
+        <v>1041</v>
       </c>
       <c r="AC133" s="3" t="n">
         <v>87338</v>
@@ -16697,7 +16697,7 @@
         <v>2163</v>
       </c>
       <c r="AB134" s="3" t="n">
-        <v>0</v>
+        <v>380</v>
       </c>
       <c r="AC134" s="3" t="n">
         <v>48581</v>
@@ -16807,7 +16807,7 @@
         <v>4555</v>
       </c>
       <c r="AB135" s="3" t="n">
-        <v>0</v>
+        <v>3296</v>
       </c>
       <c r="AC135" s="3" t="n">
         <v>81994</v>
@@ -16917,7 +16917,7 @@
         <v>828</v>
       </c>
       <c r="AB136" s="3" t="n">
-        <v>0</v>
+        <v>959</v>
       </c>
       <c r="AC136" s="3" t="n">
         <v>67674</v>
@@ -17027,7 +17027,7 @@
         <v>7893</v>
       </c>
       <c r="AB137" s="3" t="n">
-        <v>22</v>
+        <v>4712</v>
       </c>
       <c r="AC137" s="3" t="n">
         <v>115211</v>
@@ -17128,16 +17128,16 @@
         <v>0.002078</v>
       </c>
       <c r="Y138" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z138" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA138" s="3" t="n">
         <v>1844</v>
       </c>
       <c r="AB138" s="3" t="n">
-        <v>0</v>
+        <v>990</v>
       </c>
       <c r="AC138" s="3" t="n">
         <v>79850</v>
@@ -17247,7 +17247,7 @@
         <v>5438</v>
       </c>
       <c r="AB139" s="3" t="n">
-        <v>9</v>
+        <v>2742</v>
       </c>
       <c r="AC139" s="3" t="n">
         <v>122915</v>
@@ -17357,7 +17357,7 @@
         <v>980</v>
       </c>
       <c r="AB140" s="3" t="n">
-        <v>0</v>
+        <v>844</v>
       </c>
       <c r="AC140" s="3" t="n">
         <v>106840</v>
@@ -17467,7 +17467,7 @@
         <v>2411</v>
       </c>
       <c r="AB141" s="3" t="n">
-        <v>0</v>
+        <v>1196</v>
       </c>
       <c r="AC141" s="3" t="n">
         <v>50587</v>
@@ -17577,7 +17577,7 @@
         <v>1121</v>
       </c>
       <c r="AB142" s="3" t="n">
-        <v>0</v>
+        <v>1316</v>
       </c>
       <c r="AC142" s="3" t="n">
         <v>91863</v>
@@ -17687,7 +17687,7 @@
         <v>4137</v>
       </c>
       <c r="AB143" s="3" t="n">
-        <v>0</v>
+        <v>786</v>
       </c>
       <c r="AC143" s="3" t="n">
         <v>106284</v>
@@ -17797,7 +17797,7 @@
         <v>2601</v>
       </c>
       <c r="AB144" s="3" t="n">
-        <v>0</v>
+        <v>726</v>
       </c>
       <c r="AC144" s="3" t="n">
         <v>67472</v>
@@ -17907,7 +17907,7 @@
         <v>2453</v>
       </c>
       <c r="AB145" s="3" t="n">
-        <v>0</v>
+        <v>2124</v>
       </c>
       <c r="AC145" s="3" t="n">
         <v>127606</v>
@@ -18017,7 +18017,7 @@
         <v>2044</v>
       </c>
       <c r="AB146" s="3" t="n">
-        <v>0</v>
+        <v>1678</v>
       </c>
       <c r="AC146" s="3" t="n">
         <v>136782</v>
@@ -18118,7 +18118,7 @@
         <v>0.002564</v>
       </c>
       <c r="Y147" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z147" s="3" t="n">
         <v>-0</v>
@@ -18127,7 +18127,7 @@
         <v>2616</v>
       </c>
       <c r="AB147" s="3" t="n">
-        <v>0</v>
+        <v>1106</v>
       </c>
       <c r="AC147" s="3" t="n">
         <v>107078</v>
@@ -18237,7 +18237,7 @@
         <v>6956</v>
       </c>
       <c r="AB148" s="3" t="n">
-        <v>0</v>
+        <v>6744</v>
       </c>
       <c r="AC148" s="3" t="n">
         <v>111381</v>
@@ -18347,7 +18347,7 @@
         <v>2838</v>
       </c>
       <c r="AB149" s="3" t="n">
-        <v>0</v>
+        <v>554</v>
       </c>
       <c r="AC149" s="3" t="n">
         <v>70575</v>
@@ -18457,7 +18457,7 @@
         <v>3769</v>
       </c>
       <c r="AB150" s="3" t="n">
-        <v>0</v>
+        <v>527</v>
       </c>
       <c r="AC150" s="3" t="n">
         <v>55280</v>
@@ -18567,7 +18567,7 @@
         <v>5494</v>
       </c>
       <c r="AB151" s="3" t="n">
-        <v>0</v>
+        <v>5766</v>
       </c>
       <c r="AC151" s="3" t="n">
         <v>100593</v>
@@ -18668,16 +18668,16 @@
         <v>0.002351</v>
       </c>
       <c r="Y152" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z152" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA152" s="3" t="n">
         <v>1967</v>
       </c>
       <c r="AB152" s="3" t="n">
-        <v>0</v>
+        <v>653</v>
       </c>
       <c r="AC152" s="3" t="n">
         <v>92961</v>
@@ -18778,16 +18778,16 @@
         <v>0.00214</v>
       </c>
       <c r="Y153" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z153" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA153" s="3" t="n">
         <v>1559</v>
       </c>
       <c r="AB153" s="3" t="n">
-        <v>0</v>
+        <v>623</v>
       </c>
       <c r="AC153" s="3" t="n">
         <v>60461</v>
@@ -18897,7 +18897,7 @@
         <v>1141</v>
       </c>
       <c r="AB154" s="3" t="n">
-        <v>0</v>
+        <v>730</v>
       </c>
       <c r="AC154" s="3" t="n">
         <v>74109</v>
@@ -19007,7 +19007,7 @@
         <v>5986</v>
       </c>
       <c r="AB155" s="3" t="n">
-        <v>0</v>
+        <v>3523</v>
       </c>
       <c r="AC155" s="3" t="n">
         <v>89170</v>
@@ -19117,7 +19117,7 @@
         <v>704</v>
       </c>
       <c r="AB156" s="3" t="n">
-        <v>0</v>
+        <v>1924</v>
       </c>
       <c r="AC156" s="3" t="n">
         <v>116928</v>
@@ -19218,16 +19218,16 @@
         <v>0.002359</v>
       </c>
       <c r="Y157" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z157" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA157" s="3" t="n">
         <v>1949</v>
       </c>
       <c r="AB157" s="3" t="n">
-        <v>0</v>
+        <v>705</v>
       </c>
       <c r="AC157" s="3" t="n">
         <v>83749</v>
@@ -19328,16 +19328,16 @@
         <v>0.002328</v>
       </c>
       <c r="Y158" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z158" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA158" s="3" t="n">
         <v>1267</v>
       </c>
       <c r="AB158" s="3" t="n">
-        <v>0</v>
+        <v>441</v>
       </c>
       <c r="AC158" s="3" t="n">
         <v>45598</v>
@@ -19447,7 +19447,7 @@
         <v>484</v>
       </c>
       <c r="AB159" s="3" t="n">
-        <v>0</v>
+        <v>1284</v>
       </c>
       <c r="AC159" s="3" t="n">
         <v>43733</v>
@@ -19557,7 +19557,7 @@
         <v>3546</v>
       </c>
       <c r="AB160" s="3" t="n">
-        <v>0</v>
+        <v>1978</v>
       </c>
       <c r="AC160" s="3" t="n">
         <v>136770</v>
@@ -19667,7 +19667,7 @@
         <v>796</v>
       </c>
       <c r="AB161" s="3" t="n">
-        <v>0</v>
+        <v>712</v>
       </c>
       <c r="AC161" s="3" t="n">
         <v>74518</v>
@@ -19771,13 +19771,13 @@
         <v>-0</v>
       </c>
       <c r="Z162" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA162" s="3" t="n">
         <v>1727</v>
       </c>
       <c r="AB162" s="3" t="n">
-        <v>0</v>
+        <v>977</v>
       </c>
       <c r="AC162" s="3" t="n">
         <v>78300</v>
@@ -19878,16 +19878,16 @@
         <v>0.002324</v>
       </c>
       <c r="Y163" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z163" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA163" s="3" t="n">
         <v>1662</v>
       </c>
       <c r="AB163" s="3" t="n">
-        <v>0</v>
+        <v>959</v>
       </c>
       <c r="AC163" s="3" t="n">
         <v>93168</v>
@@ -19997,7 +19997,7 @@
         <v>1209</v>
       </c>
       <c r="AB164" s="3" t="n">
-        <v>0</v>
+        <v>827</v>
       </c>
       <c r="AC164" s="3" t="n">
         <v>84737</v>
@@ -20101,13 +20101,13 @@
         <v>-0</v>
       </c>
       <c r="Z165" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA165" s="3" t="n">
         <v>5041</v>
       </c>
       <c r="AB165" s="3" t="n">
-        <v>0</v>
+        <v>1673</v>
       </c>
       <c r="AC165" s="3" t="n">
         <v>111209</v>
@@ -20208,16 +20208,16 @@
         <v>0.002226</v>
       </c>
       <c r="Y166" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z166" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA166" s="3" t="n">
         <v>2856</v>
       </c>
       <c r="AB166" s="3" t="n">
-        <v>0</v>
+        <v>668</v>
       </c>
       <c r="AC166" s="3" t="n">
         <v>93034</v>
@@ -20327,7 +20327,7 @@
         <v>3166</v>
       </c>
       <c r="AB167" s="3" t="n">
-        <v>0</v>
+        <v>2741</v>
       </c>
       <c r="AC167" s="3" t="n">
         <v>140340</v>
@@ -20437,7 +20437,7 @@
         <v>8054</v>
       </c>
       <c r="AB168" s="3" t="n">
-        <v>10</v>
+        <v>2646</v>
       </c>
       <c r="AC168" s="3" t="n">
         <v>94693</v>
@@ -20547,7 +20547,7 @@
         <v>2464</v>
       </c>
       <c r="AB169" s="3" t="n">
-        <v>0</v>
+        <v>635</v>
       </c>
       <c r="AC169" s="3" t="n">
         <v>64011</v>
@@ -20657,7 +20657,7 @@
         <v>1846</v>
       </c>
       <c r="AB170" s="3" t="n">
-        <v>0</v>
+        <v>1020</v>
       </c>
       <c r="AC170" s="3" t="n">
         <v>47371</v>
@@ -20767,7 +20767,7 @@
         <v>1737</v>
       </c>
       <c r="AB171" s="3" t="n">
-        <v>0</v>
+        <v>484</v>
       </c>
       <c r="AC171" s="3" t="n">
         <v>63576</v>
@@ -20877,7 +20877,7 @@
         <v>2189</v>
       </c>
       <c r="AB172" s="3" t="n">
-        <v>0</v>
+        <v>668</v>
       </c>
       <c r="AC172" s="3" t="n">
         <v>56642</v>
@@ -20987,7 +20987,7 @@
         <v>1085</v>
       </c>
       <c r="AB173" s="3" t="n">
-        <v>0</v>
+        <v>2976</v>
       </c>
       <c r="AC173" s="3" t="n">
         <v>74782</v>
@@ -21097,7 +21097,7 @@
         <v>1727</v>
       </c>
       <c r="AB174" s="3" t="n">
-        <v>0</v>
+        <v>3090</v>
       </c>
       <c r="AC174" s="3" t="n">
         <v>134213</v>
@@ -21207,7 +21207,7 @@
         <v>1147</v>
       </c>
       <c r="AB175" s="3" t="n">
-        <v>0</v>
+        <v>905</v>
       </c>
       <c r="AC175" s="3" t="n">
         <v>62895</v>
@@ -21317,7 +21317,7 @@
         <v>1626</v>
       </c>
       <c r="AB176" s="3" t="n">
-        <v>0</v>
+        <v>1238</v>
       </c>
       <c r="AC176" s="3" t="n">
         <v>126695</v>
@@ -21427,7 +21427,7 @@
         <v>2904</v>
       </c>
       <c r="AB177" s="3" t="n">
-        <v>0</v>
+        <v>1084</v>
       </c>
       <c r="AC177" s="3" t="n">
         <v>122200</v>
@@ -21537,7 +21537,7 @@
         <v>3241</v>
       </c>
       <c r="AB178" s="3" t="n">
-        <v>0</v>
+        <v>652</v>
       </c>
       <c r="AC178" s="3" t="n">
         <v>51170</v>
@@ -21647,7 +21647,7 @@
         <v>5398</v>
       </c>
       <c r="AB179" s="3" t="n">
-        <v>0</v>
+        <v>5575</v>
       </c>
       <c r="AC179" s="3" t="n">
         <v>103555</v>
@@ -21757,7 +21757,7 @@
         <v>780</v>
       </c>
       <c r="AB180" s="3" t="n">
-        <v>0</v>
+        <v>369</v>
       </c>
       <c r="AC180" s="3" t="n">
         <v>65338</v>
@@ -21867,7 +21867,7 @@
         <v>691</v>
       </c>
       <c r="AB181" s="3" t="n">
-        <v>0</v>
+        <v>787</v>
       </c>
       <c r="AC181" s="3" t="n">
         <v>101204</v>
@@ -21977,7 +21977,7 @@
         <v>7221</v>
       </c>
       <c r="AB182" s="3" t="n">
-        <v>0</v>
+        <v>2655</v>
       </c>
       <c r="AC182" s="3" t="n">
         <v>92508</v>
@@ -22087,7 +22087,7 @@
         <v>987</v>
       </c>
       <c r="AB183" s="3" t="n">
-        <v>0</v>
+        <v>860</v>
       </c>
       <c r="AC183" s="3" t="n">
         <v>87150</v>
@@ -22197,7 +22197,7 @@
         <v>6112</v>
       </c>
       <c r="AB184" s="3" t="n">
-        <v>2</v>
+        <v>3276</v>
       </c>
       <c r="AC184" s="3" t="n">
         <v>129180</v>
@@ -22307,7 +22307,7 @@
         <v>3840</v>
       </c>
       <c r="AB185" s="3" t="n">
-        <v>0</v>
+        <v>4049</v>
       </c>
       <c r="AC185" s="3" t="n">
         <v>79248</v>
@@ -22411,13 +22411,13 @@
         <v>0</v>
       </c>
       <c r="Z186" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA186" s="3" t="n">
         <v>1460</v>
       </c>
       <c r="AB186" s="3" t="n">
-        <v>0</v>
+        <v>1734</v>
       </c>
       <c r="AC186" s="3" t="n">
         <v>92026</v>
@@ -22527,7 +22527,7 @@
         <v>963</v>
       </c>
       <c r="AB187" s="3" t="n">
-        <v>0</v>
+        <v>426</v>
       </c>
       <c r="AC187" s="3" t="n">
         <v>60331</v>
@@ -22631,13 +22631,13 @@
         <v>-0</v>
       </c>
       <c r="Z188" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA188" s="3" t="n">
         <v>1846</v>
       </c>
       <c r="AB188" s="3" t="n">
-        <v>0</v>
+        <v>928</v>
       </c>
       <c r="AC188" s="3" t="n">
         <v>75705</v>
@@ -22747,7 +22747,7 @@
         <v>572</v>
       </c>
       <c r="AB189" s="3" t="n">
-        <v>0</v>
+        <v>2789</v>
       </c>
       <c r="AC189" s="3" t="n">
         <v>43709</v>
@@ -22848,16 +22848,16 @@
         <v>0.002054</v>
       </c>
       <c r="Y190" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z190" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA190" s="3" t="n">
         <v>1712</v>
       </c>
       <c r="AB190" s="3" t="n">
-        <v>0</v>
+        <v>1635</v>
       </c>
       <c r="AC190" s="3" t="n">
         <v>134858</v>
@@ -22958,16 +22958,16 @@
         <v>0.002421</v>
       </c>
       <c r="Y191" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z191" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA191" s="3" t="n">
         <v>857</v>
       </c>
       <c r="AB191" s="3" t="n">
-        <v>0</v>
+        <v>424</v>
       </c>
       <c r="AC191" s="3" t="n">
         <v>62421</v>
@@ -23068,16 +23068,16 @@
         <v>0.001946</v>
       </c>
       <c r="Y192" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z192" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA192" s="3" t="n">
         <v>1654</v>
       </c>
       <c r="AB192" s="3" t="n">
-        <v>0</v>
+        <v>951</v>
       </c>
       <c r="AC192" s="3" t="n">
         <v>66487</v>
@@ -23187,7 +23187,7 @@
         <v>1815</v>
       </c>
       <c r="AB193" s="3" t="n">
-        <v>0</v>
+        <v>529</v>
       </c>
       <c r="AC193" s="3" t="n">
         <v>68724</v>
@@ -23297,7 +23297,7 @@
         <v>1315</v>
       </c>
       <c r="AB194" s="3" t="n">
-        <v>0</v>
+        <v>1526</v>
       </c>
       <c r="AC194" s="3" t="n">
         <v>75683</v>
@@ -23407,7 +23407,7 @@
         <v>1446</v>
       </c>
       <c r="AB195" s="3" t="n">
-        <v>0</v>
+        <v>692</v>
       </c>
       <c r="AC195" s="3" t="n">
         <v>70658</v>
@@ -23517,7 +23517,7 @@
         <v>1395</v>
       </c>
       <c r="AB196" s="3" t="n">
-        <v>0</v>
+        <v>1873</v>
       </c>
       <c r="AC196" s="3" t="n">
         <v>90787</v>
@@ -23618,7 +23618,7 @@
         <v>0.002434</v>
       </c>
       <c r="Y197" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z197" s="3" t="n">
         <v>-0</v>
@@ -23627,7 +23627,7 @@
         <v>284</v>
       </c>
       <c r="AB197" s="3" t="n">
-        <v>0</v>
+        <v>375</v>
       </c>
       <c r="AC197" s="3" t="n">
         <v>72696</v>
@@ -23737,7 +23737,7 @@
         <v>5512</v>
       </c>
       <c r="AB198" s="3" t="n">
-        <v>0</v>
+        <v>3394</v>
       </c>
       <c r="AC198" s="3" t="n">
         <v>73611</v>
@@ -23841,13 +23841,13 @@
         <v>0</v>
       </c>
       <c r="Z199" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA199" s="3" t="n">
         <v>1816</v>
       </c>
       <c r="AB199" s="3" t="n">
-        <v>0</v>
+        <v>1221</v>
       </c>
       <c r="AC199" s="3" t="n">
         <v>63703</v>
@@ -23948,7 +23948,7 @@
         <v>0.002174</v>
       </c>
       <c r="Y200" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z200" s="3" t="n">
         <v>0</v>
@@ -23957,7 +23957,7 @@
         <v>1957</v>
       </c>
       <c r="AB200" s="3" t="n">
-        <v>0</v>
+        <v>1783</v>
       </c>
       <c r="AC200" s="3" t="n">
         <v>118978</v>
@@ -24061,13 +24061,13 @@
         <v>0</v>
       </c>
       <c r="Z201" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA201" s="3" t="n">
         <v>1413</v>
       </c>
       <c r="AB201" s="3" t="n">
-        <v>0</v>
+        <v>1065</v>
       </c>
       <c r="AC201" s="3" t="n">
         <v>70248</v>
@@ -24177,7 +24177,7 @@
         <v>902</v>
       </c>
       <c r="AB202" s="3" t="n">
-        <v>0</v>
+        <v>968</v>
       </c>
       <c r="AC202" s="3" t="n">
         <v>100854</v>
@@ -24287,7 +24287,7 @@
         <v>855</v>
       </c>
       <c r="AB203" s="3" t="n">
-        <v>0</v>
+        <v>555</v>
       </c>
       <c r="AC203" s="3" t="n">
         <v>54199</v>
@@ -24397,7 +24397,7 @@
         <v>1057</v>
       </c>
       <c r="AB204" s="3" t="n">
-        <v>0</v>
+        <v>545</v>
       </c>
       <c r="AC204" s="3" t="n">
         <v>88701</v>
@@ -24507,7 +24507,7 @@
         <v>3110</v>
       </c>
       <c r="AB205" s="3" t="n">
-        <v>0</v>
+        <v>938</v>
       </c>
       <c r="AC205" s="3" t="n">
         <v>34605</v>
@@ -24608,16 +24608,16 @@
         <v>0.002336</v>
       </c>
       <c r="Y206" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z206" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA206" s="3" t="n">
         <v>1316</v>
       </c>
       <c r="AB206" s="3" t="n">
-        <v>0</v>
+        <v>1163</v>
       </c>
       <c r="AC206" s="3" t="n">
         <v>108026</v>
@@ -24721,13 +24721,13 @@
         <v>-0</v>
       </c>
       <c r="Z207" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA207" s="3" t="n">
         <v>3507</v>
       </c>
       <c r="AB207" s="3" t="n">
-        <v>0</v>
+        <v>1052</v>
       </c>
       <c r="AC207" s="3" t="n">
         <v>71665</v>
@@ -24828,16 +24828,16 @@
         <v>0.001861</v>
       </c>
       <c r="Y208" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z208" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA208" s="3" t="n">
         <v>2735</v>
       </c>
       <c r="AB208" s="3" t="n">
-        <v>0</v>
+        <v>1637</v>
       </c>
       <c r="AC208" s="3" t="n">
         <v>54773</v>
@@ -24947,7 +24947,7 @@
         <v>1086</v>
       </c>
       <c r="AB209" s="3" t="n">
-        <v>0</v>
+        <v>766</v>
       </c>
       <c r="AC209" s="3" t="n">
         <v>74745</v>
@@ -25051,13 +25051,13 @@
         <v>0</v>
       </c>
       <c r="Z210" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA210" s="3" t="n">
         <v>1407</v>
       </c>
       <c r="AB210" s="3" t="n">
-        <v>0</v>
+        <v>931</v>
       </c>
       <c r="AC210" s="3" t="n">
         <v>96872</v>
@@ -25158,16 +25158,16 @@
         <v>0.001842</v>
       </c>
       <c r="Y211" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z211" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA211" s="3" t="n">
         <v>1124</v>
       </c>
       <c r="AB211" s="3" t="n">
-        <v>0</v>
+        <v>2118</v>
       </c>
       <c r="AC211" s="3" t="n">
         <v>136683</v>
@@ -25277,7 +25277,7 @@
         <v>1359</v>
       </c>
       <c r="AB212" s="3" t="n">
-        <v>0</v>
+        <v>455</v>
       </c>
       <c r="AC212" s="3" t="n">
         <v>63555</v>
@@ -25387,7 +25387,7 @@
         <v>1611</v>
       </c>
       <c r="AB213" s="3" t="n">
-        <v>0</v>
+        <v>866</v>
       </c>
       <c r="AC213" s="3" t="n">
         <v>43936</v>
@@ -25491,13 +25491,13 @@
         <v>-0</v>
       </c>
       <c r="Z214" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA214" s="3" t="n">
         <v>952</v>
       </c>
       <c r="AB214" s="3" t="n">
-        <v>0</v>
+        <v>1489</v>
       </c>
       <c r="AC214" s="3" t="n">
         <v>91933</v>
@@ -25607,7 +25607,7 @@
         <v>759</v>
       </c>
       <c r="AB215" s="3" t="n">
-        <v>0</v>
+        <v>660</v>
       </c>
       <c r="AC215" s="3" t="n">
         <v>58675</v>
@@ -25711,13 +25711,13 @@
         <v>0</v>
       </c>
       <c r="Z216" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA216" s="3" t="n">
         <v>3049</v>
       </c>
       <c r="AB216" s="3" t="n">
-        <v>0</v>
+        <v>1011</v>
       </c>
       <c r="AC216" s="3" t="n">
         <v>68367</v>
@@ -25827,7 +25827,7 @@
         <v>2672</v>
       </c>
       <c r="AB217" s="3" t="n">
-        <v>0</v>
+        <v>927</v>
       </c>
       <c r="AC217" s="3" t="n">
         <v>53387</v>
@@ -25937,7 +25937,7 @@
         <v>2307</v>
       </c>
       <c r="AB218" s="3" t="n">
-        <v>0</v>
+        <v>3900</v>
       </c>
       <c r="AC218" s="3" t="n">
         <v>65546</v>
@@ -26047,7 +26047,7 @@
         <v>871</v>
       </c>
       <c r="AB219" s="3" t="n">
-        <v>0</v>
+        <v>639</v>
       </c>
       <c r="AC219" s="3" t="n">
         <v>57626</v>
@@ -26157,7 +26157,7 @@
         <v>720</v>
       </c>
       <c r="AB220" s="3" t="n">
-        <v>0</v>
+        <v>1095</v>
       </c>
       <c r="AC220" s="3" t="n">
         <v>84567</v>
@@ -26267,7 +26267,7 @@
         <v>1996</v>
       </c>
       <c r="AB221" s="3" t="n">
-        <v>0</v>
+        <v>408</v>
       </c>
       <c r="AC221" s="3" t="n">
         <v>39916</v>
@@ -26368,7 +26368,7 @@
         <v>0.00202</v>
       </c>
       <c r="Y222" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z222" s="3" t="n">
         <v>0</v>
@@ -26377,7 +26377,7 @@
         <v>2159</v>
       </c>
       <c r="AB222" s="3" t="n">
-        <v>0</v>
+        <v>606</v>
       </c>
       <c r="AC222" s="3" t="n">
         <v>69673</v>
@@ -26487,7 +26487,7 @@
         <v>1550</v>
       </c>
       <c r="AB223" s="3" t="n">
-        <v>0</v>
+        <v>761</v>
       </c>
       <c r="AC223" s="3" t="n">
         <v>128199</v>
@@ -26597,7 +26597,7 @@
         <v>4141</v>
       </c>
       <c r="AB224" s="3" t="n">
-        <v>0</v>
+        <v>605</v>
       </c>
       <c r="AC224" s="3" t="n">
         <v>60110</v>
@@ -26707,7 +26707,7 @@
         <v>981</v>
       </c>
       <c r="AB225" s="3" t="n">
-        <v>0</v>
+        <v>779</v>
       </c>
       <c r="AC225" s="3" t="n">
         <v>75153</v>
@@ -26817,7 +26817,7 @@
         <v>536</v>
       </c>
       <c r="AB226" s="3" t="n">
-        <v>0</v>
+        <v>490</v>
       </c>
       <c r="AC226" s="3" t="n">
         <v>42983</v>
@@ -26927,7 +26927,7 @@
         <v>1862</v>
       </c>
       <c r="AB227" s="3" t="n">
-        <v>0</v>
+        <v>359</v>
       </c>
       <c r="AC227" s="3" t="n">
         <v>67491</v>
@@ -27037,7 +27037,7 @@
         <v>1858</v>
       </c>
       <c r="AB228" s="3" t="n">
-        <v>0</v>
+        <v>1022</v>
       </c>
       <c r="AC228" s="3" t="n">
         <v>91821</v>
@@ -27147,7 +27147,7 @@
         <v>535</v>
       </c>
       <c r="AB229" s="3" t="n">
-        <v>0</v>
+        <v>1768</v>
       </c>
       <c r="AC229" s="3" t="n">
         <v>68283</v>
@@ -27251,13 +27251,13 @@
         <v>-0</v>
       </c>
       <c r="Z230" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA230" s="3" t="n">
         <v>2206</v>
       </c>
       <c r="AB230" s="3" t="n">
-        <v>0</v>
+        <v>920</v>
       </c>
       <c r="AC230" s="3" t="n">
         <v>62984</v>
@@ -27367,7 +27367,7 @@
         <v>5834</v>
       </c>
       <c r="AB231" s="3" t="n">
-        <v>0</v>
+        <v>2261</v>
       </c>
       <c r="AC231" s="3" t="n">
         <v>33739</v>
@@ -27477,7 +27477,7 @@
         <v>1275</v>
       </c>
       <c r="AB232" s="3" t="n">
-        <v>0</v>
+        <v>527</v>
       </c>
       <c r="AC232" s="3" t="n">
         <v>52652</v>
@@ -27587,7 +27587,7 @@
         <v>1699</v>
       </c>
       <c r="AB233" s="3" t="n">
-        <v>0</v>
+        <v>3247</v>
       </c>
       <c r="AC233" s="3" t="n">
         <v>69164</v>
@@ -27697,7 +27697,7 @@
         <v>941</v>
       </c>
       <c r="AB234" s="3" t="n">
-        <v>0</v>
+        <v>953</v>
       </c>
       <c r="AC234" s="3" t="n">
         <v>61371</v>
@@ -27807,7 +27807,7 @@
         <v>2347</v>
       </c>
       <c r="AB235" s="3" t="n">
-        <v>0</v>
+        <v>682</v>
       </c>
       <c r="AC235" s="3" t="n">
         <v>64779</v>
@@ -27917,7 +27917,7 @@
         <v>2201</v>
       </c>
       <c r="AB236" s="3" t="n">
-        <v>0</v>
+        <v>584</v>
       </c>
       <c r="AC236" s="3" t="n">
         <v>62172</v>
@@ -28027,7 +28027,7 @@
         <v>2918</v>
       </c>
       <c r="AB237" s="3" t="n">
-        <v>0</v>
+        <v>2975</v>
       </c>
       <c r="AC237" s="3" t="n">
         <v>47026</v>
@@ -28128,16 +28128,16 @@
         <v>0.001669</v>
       </c>
       <c r="Y238" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z238" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA238" s="3" t="n">
         <v>870</v>
       </c>
       <c r="AB238" s="3" t="n">
-        <v>0</v>
+        <v>1509</v>
       </c>
       <c r="AC238" s="3" t="n">
         <v>104437</v>
@@ -28247,7 +28247,7 @@
         <v>840</v>
       </c>
       <c r="AB239" s="3" t="n">
-        <v>0</v>
+        <v>538</v>
       </c>
       <c r="AC239" s="3" t="n">
         <v>36979</v>
@@ -28357,7 +28357,7 @@
         <v>1789</v>
       </c>
       <c r="AB240" s="3" t="n">
-        <v>0</v>
+        <v>1032</v>
       </c>
       <c r="AC240" s="3" t="n">
         <v>60443</v>
@@ -28467,7 +28467,7 @@
         <v>477</v>
       </c>
       <c r="AB241" s="3" t="n">
-        <v>0</v>
+        <v>394</v>
       </c>
       <c r="AC241" s="3" t="n">
         <v>38005</v>
@@ -28577,7 +28577,7 @@
         <v>1481</v>
       </c>
       <c r="AB242" s="3" t="n">
-        <v>0</v>
+        <v>1297</v>
       </c>
       <c r="AC242" s="3" t="n">
         <v>68993</v>
@@ -28687,7 +28687,7 @@
         <v>1538</v>
       </c>
       <c r="AB243" s="3" t="n">
-        <v>0</v>
+        <v>782</v>
       </c>
       <c r="AC243" s="3" t="n">
         <v>55330</v>
@@ -28797,7 +28797,7 @@
         <v>1390</v>
       </c>
       <c r="AB244" s="3" t="n">
-        <v>0</v>
+        <v>874</v>
       </c>
       <c r="AC244" s="3" t="n">
         <v>73112</v>
@@ -28901,13 +28901,13 @@
         <v>-0</v>
       </c>
       <c r="Z245" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA245" s="3" t="n">
         <v>552</v>
       </c>
       <c r="AB245" s="3" t="n">
-        <v>0</v>
+        <v>1098</v>
       </c>
       <c r="AC245" s="3" t="n">
         <v>66673</v>
@@ -29017,7 +29017,7 @@
         <v>673</v>
       </c>
       <c r="AB246" s="3" t="n">
-        <v>0</v>
+        <v>430</v>
       </c>
       <c r="AC246" s="3" t="n">
         <v>59627</v>
@@ -29127,7 +29127,7 @@
         <v>1931</v>
       </c>
       <c r="AB247" s="3" t="n">
-        <v>0</v>
+        <v>645</v>
       </c>
       <c r="AC247" s="3" t="n">
         <v>40995</v>
@@ -29228,16 +29228,16 @@
         <v>0.001997</v>
       </c>
       <c r="Y248" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z248" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA248" s="3" t="n">
         <v>1537</v>
       </c>
       <c r="AB248" s="3" t="n">
-        <v>0</v>
+        <v>1084</v>
       </c>
       <c r="AC248" s="3" t="n">
         <v>97317</v>
@@ -29347,7 +29347,7 @@
         <v>3225</v>
       </c>
       <c r="AB249" s="3" t="n">
-        <v>0</v>
+        <v>2383</v>
       </c>
       <c r="AC249" s="3" t="n">
         <v>39538</v>
@@ -29457,7 +29457,7 @@
         <v>1743</v>
       </c>
       <c r="AB250" s="3" t="n">
-        <v>0</v>
+        <v>494</v>
       </c>
       <c r="AC250" s="3" t="n">
         <v>82993</v>
@@ -29567,7 +29567,7 @@
         <v>887</v>
       </c>
       <c r="AB251" s="3" t="n">
-        <v>0</v>
+        <v>577</v>
       </c>
       <c r="AC251" s="3" t="n">
         <v>46558</v>
@@ -29677,7 +29677,7 @@
         <v>1259</v>
       </c>
       <c r="AB252" s="3" t="n">
-        <v>0</v>
+        <v>2935</v>
       </c>
       <c r="AC252" s="3" t="n">
         <v>79497</v>
@@ -29787,7 +29787,7 @@
         <v>1929</v>
       </c>
       <c r="AB253" s="3" t="n">
-        <v>0</v>
+        <v>617</v>
       </c>
       <c r="AC253" s="3" t="n">
         <v>77927</v>
@@ -29897,7 +29897,7 @@
         <v>544</v>
       </c>
       <c r="AB254" s="3" t="n">
-        <v>0</v>
+        <v>1286</v>
       </c>
       <c r="AC254" s="3" t="n">
         <v>71171</v>
@@ -30007,7 +30007,7 @@
         <v>1103</v>
       </c>
       <c r="AB255" s="3" t="n">
-        <v>0</v>
+        <v>543</v>
       </c>
       <c r="AC255" s="3" t="n">
         <v>91621</v>
@@ -30108,16 +30108,16 @@
         <v>0.00168</v>
       </c>
       <c r="Y256" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z256" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA256" s="3" t="n">
         <v>1090</v>
       </c>
       <c r="AB256" s="3" t="n">
-        <v>0</v>
+        <v>1606</v>
       </c>
       <c r="AC256" s="3" t="n">
         <v>55651</v>
@@ -30227,7 +30227,7 @@
         <v>1359</v>
       </c>
       <c r="AB257" s="3" t="n">
-        <v>0</v>
+        <v>3351</v>
       </c>
       <c r="AC257" s="3" t="n">
         <v>44505</v>
@@ -30337,7 +30337,7 @@
         <v>594</v>
       </c>
       <c r="AB258" s="3" t="n">
-        <v>0</v>
+        <v>961</v>
       </c>
       <c r="AC258" s="3" t="n">
         <v>77155</v>
@@ -30447,7 +30447,7 @@
         <v>1960</v>
       </c>
       <c r="AB259" s="3" t="n">
-        <v>0</v>
+        <v>443</v>
       </c>
       <c r="AC259" s="3" t="n">
         <v>39909</v>
@@ -30557,7 +30557,7 @@
         <v>1672</v>
       </c>
       <c r="AB260" s="3" t="n">
-        <v>0</v>
+        <v>1417</v>
       </c>
       <c r="AC260" s="3" t="n">
         <v>101685</v>
@@ -30667,7 +30667,7 @@
         <v>1482</v>
       </c>
       <c r="AB261" s="3" t="n">
-        <v>0</v>
+        <v>1048</v>
       </c>
       <c r="AC261" s="3" t="n">
         <v>41421</v>
@@ -30767,7 +30767,7 @@
         <v>2894</v>
       </c>
       <c r="AB262" s="3" t="n">
-        <v>0</v>
+        <v>2815</v>
       </c>
       <c r="AC262" s="3" t="n">
         <v>113705</v>
@@ -30867,7 +30867,7 @@
         <v>288</v>
       </c>
       <c r="AB263" s="3" t="n">
-        <v>0</v>
+        <v>548</v>
       </c>
       <c r="AC263" s="3" t="n">
         <v>54482</v>
@@ -30967,7 +30967,7 @@
         <v>3713</v>
       </c>
       <c r="AB264" s="3" t="n">
-        <v>0</v>
+        <v>471</v>
       </c>
       <c r="AC264" s="3" t="n">
         <v>42174</v>
@@ -31067,7 +31067,7 @@
         <v>999</v>
       </c>
       <c r="AB265" s="3" t="n">
-        <v>0</v>
+        <v>415</v>
       </c>
       <c r="AC265" s="3" t="n">
         <v>55367</v>
@@ -31167,7 +31167,7 @@
         <v>1523</v>
       </c>
       <c r="AB266" s="3" t="n">
-        <v>0</v>
+        <v>446</v>
       </c>
       <c r="AC266" s="3" t="n">
         <v>59123</v>
@@ -31267,7 +31267,7 @@
         <v>916</v>
       </c>
       <c r="AB267" s="3" t="n">
-        <v>0</v>
+        <v>1012</v>
       </c>
       <c r="AC267" s="3" t="n">
         <v>47987</v>
@@ -31367,7 +31367,7 @@
         <v>867</v>
       </c>
       <c r="AB268" s="3" t="n">
-        <v>0</v>
+        <v>1145</v>
       </c>
       <c r="AC268" s="3" t="n">
         <v>59025</v>
@@ -31467,7 +31467,7 @@
         <v>2071</v>
       </c>
       <c r="AB269" s="3" t="n">
-        <v>0</v>
+        <v>5690</v>
       </c>
       <c r="AC269" s="3" t="n">
         <v>78384</v>
@@ -31558,16 +31558,16 @@
         <v>0.002001</v>
       </c>
       <c r="Y270" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z270" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA270" s="3" t="n">
         <v>692</v>
       </c>
       <c r="AB270" s="3" t="n">
-        <v>0</v>
+        <v>1569</v>
       </c>
       <c r="AC270" s="3" t="n">
         <v>78132</v>
@@ -31667,7 +31667,7 @@
         <v>1315</v>
       </c>
       <c r="AB271" s="3" t="n">
-        <v>0</v>
+        <v>1149</v>
       </c>
       <c r="AC271" s="3" t="n">
         <v>64961</v>
@@ -31767,7 +31767,7 @@
         <v>1466</v>
       </c>
       <c r="AB272" s="3" t="n">
-        <v>0</v>
+        <v>1484</v>
       </c>
       <c r="AC272" s="3" t="n">
         <v>38083</v>
@@ -31867,7 +31867,7 @@
         <v>489</v>
       </c>
       <c r="AB273" s="3" t="n">
-        <v>0</v>
+        <v>584</v>
       </c>
       <c r="AC273" s="3" t="n">
         <v>57213</v>
@@ -31967,7 +31967,7 @@
         <v>3118</v>
       </c>
       <c r="AB274" s="3" t="n">
-        <v>0</v>
+        <v>796</v>
       </c>
       <c r="AC274" s="3" t="n">
         <v>83239</v>
@@ -32067,7 +32067,7 @@
         <v>1615</v>
       </c>
       <c r="AB275" s="3" t="n">
-        <v>0</v>
+        <v>547</v>
       </c>
       <c r="AC275" s="3" t="n">
         <v>52585</v>
@@ -32158,16 +32158,16 @@
         <v>0.001928</v>
       </c>
       <c r="Y276" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z276" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA276" s="3" t="n">
         <v>348</v>
       </c>
       <c r="AB276" s="3" t="n">
-        <v>0</v>
+        <v>418</v>
       </c>
       <c r="AC276" s="3" t="n">
         <v>60145</v>
@@ -32267,7 +32267,7 @@
         <v>1212</v>
       </c>
       <c r="AB277" s="3" t="n">
-        <v>0</v>
+        <v>543</v>
       </c>
       <c r="AC277" s="3" t="n">
         <v>61083</v>
@@ -32367,7 +32367,7 @@
         <v>2825</v>
       </c>
       <c r="AB278" s="3" t="n">
-        <v>0</v>
+        <v>520</v>
       </c>
       <c r="AC278" s="3" t="n">
         <v>43582</v>
@@ -32467,7 +32467,7 @@
         <v>1102</v>
       </c>
       <c r="AB279" s="3" t="n">
-        <v>0</v>
+        <v>635</v>
       </c>
       <c r="AC279" s="3" t="n">
         <v>67633</v>
@@ -32561,13 +32561,13 @@
         <v>-0</v>
       </c>
       <c r="Z280" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA280" s="3" t="n">
         <v>745</v>
       </c>
       <c r="AB280" s="3" t="n">
-        <v>0</v>
+        <v>839</v>
       </c>
       <c r="AC280" s="3" t="n">
         <v>69534</v>
@@ -32667,7 +32667,7 @@
         <v>1174</v>
       </c>
       <c r="AB281" s="3" t="n">
-        <v>0</v>
+        <v>1097</v>
       </c>
       <c r="AC281" s="3" t="n">
         <v>70693</v>
@@ -32761,13 +32761,13 @@
         <v>-0</v>
       </c>
       <c r="Z282" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA282" s="3" t="n">
         <v>2005</v>
       </c>
       <c r="AB282" s="3" t="n">
-        <v>0</v>
+        <v>609</v>
       </c>
       <c r="AC282" s="3" t="n">
         <v>76021</v>
@@ -32867,7 +32867,7 @@
         <v>4625</v>
       </c>
       <c r="AB283" s="3" t="n">
-        <v>0</v>
+        <v>2269</v>
       </c>
       <c r="AC283" s="3" t="n">
         <v>99588</v>
@@ -32967,7 +32967,7 @@
         <v>497</v>
       </c>
       <c r="AB284" s="3" t="n">
-        <v>0</v>
+        <v>728</v>
       </c>
       <c r="AC284" s="3" t="n">
         <v>63750</v>
@@ -33067,7 +33067,7 @@
         <v>521</v>
       </c>
       <c r="AB285" s="3" t="n">
-        <v>0</v>
+        <v>485</v>
       </c>
       <c r="AC285" s="3" t="n">
         <v>69396</v>
@@ -33161,13 +33161,13 @@
         <v>0</v>
       </c>
       <c r="Z286" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA286" s="3" t="n">
         <v>627</v>
       </c>
       <c r="AB286" s="3" t="n">
-        <v>0</v>
+        <v>784</v>
       </c>
       <c r="AC286" s="3" t="n">
         <v>48014</v>
@@ -33267,7 +33267,7 @@
         <v>2337</v>
       </c>
       <c r="AB287" s="3" t="n">
-        <v>0</v>
+        <v>1167</v>
       </c>
       <c r="AC287" s="3" t="n">
         <v>86970</v>
@@ -33367,7 +33367,7 @@
         <v>1436</v>
       </c>
       <c r="AB288" s="3" t="n">
-        <v>0</v>
+        <v>409</v>
       </c>
       <c r="AC288" s="3" t="n">
         <v>47848</v>
@@ -33467,7 +33467,7 @@
         <v>3450</v>
       </c>
       <c r="AB289" s="3" t="n">
-        <v>0</v>
+        <v>826</v>
       </c>
       <c r="AC289" s="3" t="n">
         <v>61636</v>
@@ -33567,7 +33567,7 @@
         <v>572</v>
       </c>
       <c r="AB290" s="3" t="n">
-        <v>0</v>
+        <v>1128</v>
       </c>
       <c r="AC290" s="3" t="n">
         <v>56996</v>
@@ -33661,13 +33661,13 @@
         <v>0</v>
       </c>
       <c r="Z291" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA291" s="3" t="n">
         <v>1844</v>
       </c>
       <c r="AB291" s="3" t="n">
-        <v>0</v>
+        <v>956</v>
       </c>
       <c r="AC291" s="3" t="n">
         <v>45222</v>
@@ -33767,7 +33767,7 @@
         <v>1150</v>
       </c>
       <c r="AB292" s="3" t="n">
-        <v>0</v>
+        <v>1464</v>
       </c>
       <c r="AC292" s="3" t="n">
         <v>34432</v>
@@ -33867,7 +33867,7 @@
         <v>313</v>
       </c>
       <c r="AB293" s="3" t="n">
-        <v>0</v>
+        <v>472</v>
       </c>
       <c r="AC293" s="3" t="n">
         <v>65922</v>
@@ -33967,7 +33967,7 @@
         <v>3348</v>
       </c>
       <c r="AB294" s="3" t="n">
-        <v>0</v>
+        <v>3743</v>
       </c>
       <c r="AC294" s="3" t="n">
         <v>86029</v>
@@ -34067,7 +34067,7 @@
         <v>941</v>
       </c>
       <c r="AB295" s="3" t="n">
-        <v>0</v>
+        <v>815</v>
       </c>
       <c r="AC295" s="3" t="n">
         <v>45453</v>
@@ -34167,7 +34167,7 @@
         <v>1622</v>
       </c>
       <c r="AB296" s="3" t="n">
-        <v>0</v>
+        <v>1158</v>
       </c>
       <c r="AC296" s="3" t="n">
         <v>72098</v>
@@ -34267,7 +34267,7 @@
         <v>841</v>
       </c>
       <c r="AB297" s="3" t="n">
-        <v>0</v>
+        <v>757</v>
       </c>
       <c r="AC297" s="3" t="n">
         <v>68874</v>
@@ -34367,7 +34367,7 @@
         <v>2294</v>
       </c>
       <c r="AB298" s="3" t="n">
-        <v>0</v>
+        <v>1043</v>
       </c>
       <c r="AC298" s="3" t="n">
         <v>82908</v>
@@ -34467,7 +34467,7 @@
         <v>1923</v>
       </c>
       <c r="AB299" s="3" t="n">
-        <v>0</v>
+        <v>677</v>
       </c>
       <c r="AC299" s="3" t="n">
         <v>52529</v>
@@ -34567,7 +34567,7 @@
         <v>786</v>
       </c>
       <c r="AB300" s="3" t="n">
-        <v>0</v>
+        <v>1339</v>
       </c>
       <c r="AC300" s="3" t="n">
         <v>52905</v>
@@ -34667,7 +34667,7 @@
         <v>1455</v>
       </c>
       <c r="AB301" s="3" t="n">
-        <v>0</v>
+        <v>3562</v>
       </c>
       <c r="AC301" s="3" t="n">
         <v>40510</v>
@@ -34767,7 +34767,7 @@
         <v>902</v>
       </c>
       <c r="AB302" s="3" t="n">
-        <v>0</v>
+        <v>1273</v>
       </c>
       <c r="AC302" s="3" t="n">
         <v>88163</v>
@@ -34867,7 +34867,7 @@
         <v>689</v>
       </c>
       <c r="AB303" s="3" t="n">
-        <v>0</v>
+        <v>1609</v>
       </c>
       <c r="AC303" s="3" t="n">
         <v>87906</v>
@@ -34967,7 +34967,7 @@
         <v>1358</v>
       </c>
       <c r="AB304" s="3" t="n">
-        <v>0</v>
+        <v>1770</v>
       </c>
       <c r="AC304" s="3" t="n">
         <v>46334</v>
@@ -35067,7 +35067,7 @@
         <v>346</v>
       </c>
       <c r="AB305" s="3" t="n">
-        <v>0</v>
+        <v>2675</v>
       </c>
       <c r="AC305" s="3" t="n">
         <v>48721</v>
@@ -35167,7 +35167,7 @@
         <v>205</v>
       </c>
       <c r="AB306" s="3" t="n">
-        <v>0</v>
+        <v>494</v>
       </c>
       <c r="AC306" s="3" t="n">
         <v>33998</v>
@@ -35258,7 +35258,7 @@
         <v>0.001379</v>
       </c>
       <c r="Y307" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z307" s="3" t="n">
         <v>0</v>
@@ -35267,7 +35267,7 @@
         <v>1535</v>
       </c>
       <c r="AB307" s="3" t="n">
-        <v>0</v>
+        <v>1140</v>
       </c>
       <c r="AC307" s="3" t="n">
         <v>59415</v>
@@ -35367,7 +35367,7 @@
         <v>3558</v>
       </c>
       <c r="AB308" s="3" t="n">
-        <v>0</v>
+        <v>1425</v>
       </c>
       <c r="AC308" s="3" t="n">
         <v>35418</v>
@@ -35467,7 +35467,7 @@
         <v>743</v>
       </c>
       <c r="AB309" s="3" t="n">
-        <v>0</v>
+        <v>1203</v>
       </c>
       <c r="AC309" s="3" t="n">
         <v>80946</v>
@@ -35567,7 +35567,7 @@
         <v>877</v>
       </c>
       <c r="AB310" s="3" t="n">
-        <v>0</v>
+        <v>912</v>
       </c>
       <c r="AC310" s="3" t="n">
         <v>41042</v>
@@ -35667,7 +35667,7 @@
         <v>1321</v>
       </c>
       <c r="AB311" s="3" t="n">
-        <v>0</v>
+        <v>1069</v>
       </c>
       <c r="AC311" s="3" t="n">
         <v>39461</v>
@@ -35767,7 +35767,7 @@
         <v>404</v>
       </c>
       <c r="AB312" s="3" t="n">
-        <v>0</v>
+        <v>567</v>
       </c>
       <c r="AC312" s="3" t="n">
         <v>47175</v>
@@ -35867,7 +35867,7 @@
         <v>627</v>
       </c>
       <c r="AB313" s="3" t="n">
-        <v>0</v>
+        <v>531</v>
       </c>
       <c r="AC313" s="3" t="n">
         <v>51097</v>
@@ -35967,7 +35967,7 @@
         <v>1829</v>
       </c>
       <c r="AB314" s="3" t="n">
-        <v>0</v>
+        <v>644</v>
       </c>
       <c r="AC314" s="3" t="n">
         <v>77339</v>
@@ -36058,16 +36058,16 @@
         <v>0.001896</v>
       </c>
       <c r="Y315" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z315" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA315" s="3" t="n">
         <v>1537</v>
       </c>
       <c r="AB315" s="3" t="n">
-        <v>0</v>
+        <v>921</v>
       </c>
       <c r="AC315" s="3" t="n">
         <v>62179</v>
@@ -36167,7 +36167,7 @@
         <v>6019</v>
       </c>
       <c r="AB316" s="3" t="n">
-        <v>0</v>
+        <v>3266</v>
       </c>
       <c r="AC316" s="3" t="n">
         <v>54909</v>
@@ -36267,7 +36267,7 @@
         <v>778</v>
       </c>
       <c r="AB317" s="3" t="n">
-        <v>0</v>
+        <v>481</v>
       </c>
       <c r="AC317" s="3" t="n">
         <v>52021</v>
@@ -36361,13 +36361,13 @@
         <v>0</v>
       </c>
       <c r="Z318" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA318" s="3" t="n">
         <v>800</v>
       </c>
       <c r="AB318" s="3" t="n">
-        <v>0</v>
+        <v>801</v>
       </c>
       <c r="AC318" s="3" t="n">
         <v>55623</v>
@@ -36467,7 +36467,7 @@
         <v>209</v>
       </c>
       <c r="AB319" s="3" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="AC319" s="3" t="n">
         <v>29697</v>
@@ -36567,7 +36567,7 @@
         <v>569</v>
       </c>
       <c r="AB320" s="3" t="n">
-        <v>0</v>
+        <v>355</v>
       </c>
       <c r="AC320" s="3" t="n">
         <v>41715</v>
@@ -36667,7 +36667,7 @@
         <v>1854</v>
       </c>
       <c r="AB321" s="3" t="n">
-        <v>0</v>
+        <v>1310</v>
       </c>
       <c r="AC321" s="3" t="n">
         <v>25407</v>
@@ -36767,7 +36767,7 @@
         <v>211</v>
       </c>
       <c r="AB322" s="3" t="n">
-        <v>0</v>
+        <v>473</v>
       </c>
       <c r="AC322" s="3" t="n">
         <v>45993</v>
@@ -36867,7 +36867,7 @@
         <v>2054</v>
       </c>
       <c r="AB323" s="3" t="n">
-        <v>0</v>
+        <v>555</v>
       </c>
       <c r="AC323" s="3" t="n">
         <v>53750</v>
@@ -36967,7 +36967,7 @@
         <v>2274</v>
       </c>
       <c r="AB324" s="3" t="n">
-        <v>0</v>
+        <v>2027</v>
       </c>
       <c r="AC324" s="3" t="n">
         <v>30737</v>
@@ -37061,13 +37061,13 @@
         <v>0</v>
       </c>
       <c r="Z325" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA325" s="3" t="n">
         <v>953</v>
       </c>
       <c r="AB325" s="3" t="n">
-        <v>0</v>
+        <v>1209</v>
       </c>
       <c r="AC325" s="3" t="n">
         <v>49942</v>
@@ -37167,7 +37167,7 @@
         <v>1613</v>
       </c>
       <c r="AB326" s="3" t="n">
-        <v>0</v>
+        <v>1703</v>
       </c>
       <c r="AC326" s="3" t="n">
         <v>58766</v>
@@ -37267,7 +37267,7 @@
         <v>481</v>
       </c>
       <c r="AB327" s="3" t="n">
-        <v>0</v>
+        <v>768</v>
       </c>
       <c r="AC327" s="3" t="n">
         <v>56816</v>
@@ -37361,13 +37361,13 @@
         <v>0</v>
       </c>
       <c r="Z328" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA328" s="3" t="n">
         <v>2839</v>
       </c>
       <c r="AB328" s="3" t="n">
-        <v>0</v>
+        <v>564</v>
       </c>
       <c r="AC328" s="3" t="n">
         <v>27253</v>
@@ -37467,7 +37467,7 @@
         <v>1523</v>
       </c>
       <c r="AB329" s="3" t="n">
-        <v>0</v>
+        <v>1859</v>
       </c>
       <c r="AC329" s="3" t="n">
         <v>28413</v>
@@ -37567,7 +37567,7 @@
         <v>849</v>
       </c>
       <c r="AB330" s="3" t="n">
-        <v>0</v>
+        <v>1257</v>
       </c>
       <c r="AC330" s="3" t="n">
         <v>36336</v>
@@ -37667,7 +37667,7 @@
         <v>669</v>
       </c>
       <c r="AB331" s="3" t="n">
-        <v>0</v>
+        <v>862</v>
       </c>
       <c r="AC331" s="3" t="n">
         <v>58667</v>
@@ -37767,7 +37767,7 @@
         <v>716</v>
       </c>
       <c r="AB332" s="3" t="n">
-        <v>0</v>
+        <v>1159</v>
       </c>
       <c r="AC332" s="3" t="n">
         <v>28712</v>
@@ -37867,7 +37867,7 @@
         <v>3008</v>
       </c>
       <c r="AB333" s="3" t="n">
-        <v>0</v>
+        <v>1591</v>
       </c>
       <c r="AC333" s="3" t="n">
         <v>95059</v>
@@ -37967,7 +37967,7 @@
         <v>211</v>
       </c>
       <c r="AB334" s="3" t="n">
-        <v>0</v>
+        <v>565</v>
       </c>
       <c r="AC334" s="3" t="n">
         <v>20661</v>
@@ -38067,7 +38067,7 @@
         <v>1180</v>
       </c>
       <c r="AB335" s="3" t="n">
-        <v>0</v>
+        <v>841</v>
       </c>
       <c r="AC335" s="3" t="n">
         <v>48434</v>
@@ -38167,7 +38167,7 @@
         <v>1230</v>
       </c>
       <c r="AB336" s="3" t="n">
-        <v>0</v>
+        <v>2094</v>
       </c>
       <c r="AC336" s="3" t="n">
         <v>54328</v>
@@ -38267,7 +38267,7 @@
         <v>1917</v>
       </c>
       <c r="AB337" s="3" t="n">
-        <v>0</v>
+        <v>2142</v>
       </c>
       <c r="AC337" s="3" t="n">
         <v>85340</v>
@@ -38367,7 +38367,7 @@
         <v>2186</v>
       </c>
       <c r="AB338" s="3" t="n">
-        <v>0</v>
+        <v>1653</v>
       </c>
       <c r="AC338" s="3" t="n">
         <v>27549</v>
@@ -38467,7 +38467,7 @@
         <v>1058</v>
       </c>
       <c r="AB339" s="3" t="n">
-        <v>0</v>
+        <v>308</v>
       </c>
       <c r="AC339" s="3" t="n">
         <v>36599</v>
@@ -38558,7 +38558,7 @@
         <v>0.001476</v>
       </c>
       <c r="Y340" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z340" s="3" t="n">
         <v>-0</v>
@@ -38567,7 +38567,7 @@
         <v>556</v>
       </c>
       <c r="AB340" s="3" t="n">
-        <v>0</v>
+        <v>494</v>
       </c>
       <c r="AC340" s="3" t="n">
         <v>39874</v>
@@ -38667,7 +38667,7 @@
         <v>1249</v>
       </c>
       <c r="AB341" s="3" t="n">
-        <v>0</v>
+        <v>1391</v>
       </c>
       <c r="AC341" s="3" t="n">
         <v>54650</v>
@@ -38767,7 +38767,7 @@
         <v>1307</v>
       </c>
       <c r="AB342" s="3" t="n">
-        <v>0</v>
+        <v>2732</v>
       </c>
       <c r="AC342" s="3" t="n">
         <v>82450</v>
@@ -38867,7 +38867,7 @@
         <v>696</v>
       </c>
       <c r="AB343" s="3" t="n">
-        <v>0</v>
+        <v>627</v>
       </c>
       <c r="AC343" s="3" t="n">
         <v>40035</v>
@@ -38967,7 +38967,7 @@
         <v>1831</v>
       </c>
       <c r="AB344" s="3" t="n">
-        <v>0</v>
+        <v>907</v>
       </c>
       <c r="AC344" s="3" t="n">
         <v>64936</v>
@@ -39067,7 +39067,7 @@
         <v>955</v>
       </c>
       <c r="AB345" s="3" t="n">
-        <v>0</v>
+        <v>565</v>
       </c>
       <c r="AC345" s="3" t="n">
         <v>54049</v>
@@ -39167,7 +39167,7 @@
         <v>105</v>
       </c>
       <c r="AB346" s="3" t="n">
-        <v>0</v>
+        <v>571</v>
       </c>
       <c r="AC346" s="3" t="n">
         <v>48660</v>
@@ -39267,7 +39267,7 @@
         <v>1161</v>
       </c>
       <c r="AB347" s="3" t="n">
-        <v>0</v>
+        <v>551</v>
       </c>
       <c r="AC347" s="3" t="n">
         <v>55682</v>
@@ -39361,13 +39361,13 @@
         <v>0</v>
       </c>
       <c r="Z348" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA348" s="3" t="n">
         <v>1209</v>
       </c>
       <c r="AB348" s="3" t="n">
-        <v>0</v>
+        <v>1175</v>
       </c>
       <c r="AC348" s="3" t="n">
         <v>49166</v>
@@ -39467,7 +39467,7 @@
         <v>1046</v>
       </c>
       <c r="AB349" s="3" t="n">
-        <v>0</v>
+        <v>771</v>
       </c>
       <c r="AC349" s="3" t="n">
         <v>41700</v>
@@ -39567,7 +39567,7 @@
         <v>2560</v>
       </c>
       <c r="AB350" s="3" t="n">
-        <v>0</v>
+        <v>3334</v>
       </c>
       <c r="AC350" s="3" t="n">
         <v>42141</v>
@@ -39667,7 +39667,7 @@
         <v>1190</v>
       </c>
       <c r="AB351" s="3" t="n">
-        <v>0</v>
+        <v>1070</v>
       </c>
       <c r="AC351" s="3" t="n">
         <v>28949</v>
@@ -39761,13 +39761,13 @@
         <v>0</v>
       </c>
       <c r="Z352" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA352" s="3" t="n">
         <v>2349</v>
       </c>
       <c r="AB352" s="3" t="n">
-        <v>0</v>
+        <v>1055</v>
       </c>
       <c r="AC352" s="3" t="n">
         <v>51041</v>
@@ -39858,16 +39858,16 @@
         <v>0.001561</v>
       </c>
       <c r="Y353" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z353" s="3" t="n">
         <v>-0</v>
-      </c>
-      <c r="Z353" s="3" t="n">
-        <v>0</v>
       </c>
       <c r="AA353" s="3" t="n">
         <v>887</v>
       </c>
       <c r="AB353" s="3" t="n">
-        <v>0</v>
+        <v>799</v>
       </c>
       <c r="AC353" s="3" t="n">
         <v>70274</v>
@@ -39958,16 +39958,16 @@
         <v>0.001581</v>
       </c>
       <c r="Y354" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z354" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA354" s="3" t="n">
         <v>1125</v>
       </c>
       <c r="AB354" s="3" t="n">
-        <v>0</v>
+        <v>749</v>
       </c>
       <c r="AC354" s="3" t="n">
         <v>72720</v>
@@ -40067,7 +40067,7 @@
         <v>3541</v>
       </c>
       <c r="AB355" s="3" t="n">
-        <v>0</v>
+        <v>2267</v>
       </c>
       <c r="AC355" s="3" t="n">
         <v>36088</v>
@@ -40167,7 +40167,7 @@
         <v>2076</v>
       </c>
       <c r="AB356" s="3" t="n">
-        <v>0</v>
+        <v>1741</v>
       </c>
       <c r="AC356" s="3" t="n">
         <v>71766</v>
@@ -40267,7 +40267,7 @@
         <v>651</v>
       </c>
       <c r="AB357" s="3" t="n">
-        <v>0</v>
+        <v>338</v>
       </c>
       <c r="AC357" s="3" t="n">
         <v>48555</v>
@@ -40367,7 +40367,7 @@
         <v>3739</v>
       </c>
       <c r="AB358" s="3" t="n">
-        <v>0</v>
+        <v>1637</v>
       </c>
       <c r="AC358" s="3" t="n">
         <v>41701</v>
@@ -40458,16 +40458,16 @@
         <v>0.00144</v>
       </c>
       <c r="Y359" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z359" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA359" s="3" t="n">
         <v>622</v>
       </c>
       <c r="AB359" s="3" t="n">
-        <v>0</v>
+        <v>1349</v>
       </c>
       <c r="AC359" s="3" t="n">
         <v>85402</v>
@@ -40567,7 +40567,7 @@
         <v>527</v>
       </c>
       <c r="AB360" s="3" t="n">
-        <v>0</v>
+        <v>963</v>
       </c>
       <c r="AC360" s="3" t="n">
         <v>52987</v>
@@ -40667,7 +40667,7 @@
         <v>84</v>
       </c>
       <c r="AB361" s="3" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="AC361" s="3" t="n">
         <v>35343</v>
@@ -40767,7 +40767,7 @@
         <v>771</v>
       </c>
       <c r="AB362" s="3" t="n">
-        <v>0</v>
+        <v>1620</v>
       </c>
       <c r="AC362" s="3" t="n">
         <v>37740</v>
@@ -40867,7 +40867,7 @@
         <v>271</v>
       </c>
       <c r="AB363" s="3" t="n">
-        <v>0</v>
+        <v>695</v>
       </c>
       <c r="AC363" s="3" t="n">
         <v>53906</v>
@@ -40967,7 +40967,7 @@
         <v>708</v>
       </c>
       <c r="AB364" s="3" t="n">
-        <v>0</v>
+        <v>761</v>
       </c>
       <c r="AC364" s="3" t="n">
         <v>40611</v>
@@ -41061,13 +41061,13 @@
         <v>0</v>
       </c>
       <c r="Z365" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA365" s="3" t="n">
         <v>1348</v>
       </c>
       <c r="AB365" s="3" t="n">
-        <v>0</v>
+        <v>624</v>
       </c>
       <c r="AC365" s="3" t="n">
         <v>80276</v>
@@ -41167,7 +41167,7 @@
         <v>740</v>
       </c>
       <c r="AB366" s="3" t="n">
-        <v>0</v>
+        <v>1307</v>
       </c>
       <c r="AC366" s="3" t="n">
         <v>42958</v>
@@ -41267,7 +41267,7 @@
         <v>3110</v>
       </c>
       <c r="AB367" s="3" t="n">
-        <v>0</v>
+        <v>1687</v>
       </c>
       <c r="AC367" s="3" t="n">
         <v>79585</v>
@@ -41367,7 +41367,7 @@
         <v>761</v>
       </c>
       <c r="AB368" s="3" t="n">
-        <v>0</v>
+        <v>182</v>
       </c>
       <c r="AC368" s="3" t="n">
         <v>23917</v>
@@ -41467,7 +41467,7 @@
         <v>1466</v>
       </c>
       <c r="AB369" s="3" t="n">
-        <v>0</v>
+        <v>290</v>
       </c>
       <c r="AC369" s="3" t="n">
         <v>23524</v>
@@ -41567,7 +41567,7 @@
         <v>783</v>
       </c>
       <c r="AB370" s="3" t="n">
-        <v>0</v>
+        <v>1121</v>
       </c>
       <c r="AC370" s="3" t="n">
         <v>49816</v>
@@ -41667,7 +41667,7 @@
         <v>372</v>
       </c>
       <c r="AB371" s="3" t="n">
-        <v>0</v>
+        <v>169</v>
       </c>
       <c r="AC371" s="3" t="n">
         <v>36022</v>
@@ -41767,7 +41767,7 @@
         <v>1418</v>
       </c>
       <c r="AB372" s="3" t="n">
-        <v>0</v>
+        <v>189</v>
       </c>
       <c r="AC372" s="3" t="n">
         <v>23881</v>
@@ -41867,7 +41867,7 @@
         <v>1934</v>
       </c>
       <c r="AB373" s="3" t="n">
-        <v>0</v>
+        <v>1829</v>
       </c>
       <c r="AC373" s="3" t="n">
         <v>52072</v>
@@ -41967,7 +41967,7 @@
         <v>159</v>
       </c>
       <c r="AB374" s="3" t="n">
-        <v>0</v>
+        <v>396</v>
       </c>
       <c r="AC374" s="3" t="n">
         <v>37898</v>
@@ -42058,7 +42058,7 @@
         <v>0.000982</v>
       </c>
       <c r="Y375" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z375" s="3" t="n">
         <v>0</v>
@@ -42067,7 +42067,7 @@
         <v>1642</v>
       </c>
       <c r="AB375" s="3" t="n">
-        <v>0</v>
+        <v>677</v>
       </c>
       <c r="AC375" s="3" t="n">
         <v>36062</v>
@@ -42167,7 +42167,7 @@
         <v>1235</v>
       </c>
       <c r="AB376" s="3" t="n">
-        <v>0</v>
+        <v>119</v>
       </c>
       <c r="AC376" s="3" t="n">
         <v>20826</v>
@@ -42267,7 +42267,7 @@
         <v>272</v>
       </c>
       <c r="AB377" s="3" t="n">
-        <v>0</v>
+        <v>303</v>
       </c>
       <c r="AC377" s="3" t="n">
         <v>29349</v>
@@ -42367,7 +42367,7 @@
         <v>343</v>
       </c>
       <c r="AB378" s="3" t="n">
-        <v>0</v>
+        <v>176</v>
       </c>
       <c r="AC378" s="3" t="n">
         <v>35423</v>
@@ -42467,7 +42467,7 @@
         <v>293</v>
       </c>
       <c r="AB379" s="3" t="n">
-        <v>0</v>
+        <v>1128</v>
       </c>
       <c r="AC379" s="3" t="n">
         <v>32649</v>
@@ -42567,7 +42567,7 @@
         <v>792</v>
       </c>
       <c r="AB380" s="3" t="n">
-        <v>0</v>
+        <v>688</v>
       </c>
       <c r="AC380" s="3" t="n">
         <v>30764</v>
@@ -42667,7 +42667,7 @@
         <v>330</v>
       </c>
       <c r="AB381" s="3" t="n">
-        <v>0</v>
+        <v>353</v>
       </c>
       <c r="AC381" s="3" t="n">
         <v>16300</v>
@@ -42767,7 +42767,7 @@
         <v>1161</v>
       </c>
       <c r="AB382" s="3" t="n">
-        <v>0</v>
+        <v>556</v>
       </c>
       <c r="AC382" s="3" t="n">
         <v>31327</v>
@@ -42858,16 +42858,16 @@
         <v>0.001105</v>
       </c>
       <c r="Y383" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z383" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA383" s="3" t="n">
         <v>247</v>
       </c>
       <c r="AB383" s="3" t="n">
-        <v>0</v>
+        <v>713</v>
       </c>
       <c r="AC383" s="3" t="n">
         <v>54026</v>
@@ -42961,13 +42961,13 @@
         <v>0</v>
       </c>
       <c r="Z384" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA384" s="3" t="n">
         <v>242</v>
       </c>
       <c r="AB384" s="3" t="n">
-        <v>0</v>
+        <v>411</v>
       </c>
       <c r="AC384" s="3" t="n">
         <v>21057</v>
@@ -43067,7 +43067,7 @@
         <v>447</v>
       </c>
       <c r="AB385" s="3" t="n">
-        <v>0</v>
+        <v>465</v>
       </c>
       <c r="AC385" s="3" t="n">
         <v>13209</v>
@@ -43167,7 +43167,7 @@
         <v>380</v>
       </c>
       <c r="AB386" s="3" t="n">
-        <v>0</v>
+        <v>460</v>
       </c>
       <c r="AC386" s="3" t="n">
         <v>22787</v>
@@ -43258,16 +43258,16 @@
         <v>0.001156</v>
       </c>
       <c r="Y387" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z387" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA387" s="3" t="n">
         <v>607</v>
       </c>
       <c r="AB387" s="3" t="n">
-        <v>0</v>
+        <v>1020</v>
       </c>
       <c r="AC387" s="3" t="n">
         <v>51469</v>
@@ -43367,7 +43367,7 @@
         <v>247</v>
       </c>
       <c r="AB388" s="3" t="n">
-        <v>0</v>
+        <v>269</v>
       </c>
       <c r="AC388" s="3" t="n">
         <v>22229</v>
@@ -43461,13 +43461,13 @@
         <v>0</v>
       </c>
       <c r="Z389" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA389" s="3" t="n">
         <v>502</v>
       </c>
       <c r="AB389" s="3" t="n">
-        <v>0</v>
+        <v>304</v>
       </c>
       <c r="AC389" s="3" t="n">
         <v>24122</v>
@@ -43567,7 +43567,7 @@
         <v>451</v>
       </c>
       <c r="AB390" s="3" t="n">
-        <v>0</v>
+        <v>783</v>
       </c>
       <c r="AC390" s="3" t="n">
         <v>32150</v>
@@ -43658,7 +43658,7 @@
         <v>0.00102</v>
       </c>
       <c r="Y391" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z391" s="3" t="n">
         <v>0</v>
@@ -43667,7 +43667,7 @@
         <v>230</v>
       </c>
       <c r="AB391" s="3" t="n">
-        <v>0</v>
+        <v>166</v>
       </c>
       <c r="AC391" s="3" t="n">
         <v>22069</v>
@@ -43767,7 +43767,7 @@
         <v>643</v>
       </c>
       <c r="AB392" s="3" t="n">
-        <v>0</v>
+        <v>615</v>
       </c>
       <c r="AC392" s="3" t="n">
         <v>29921</v>
@@ -43861,13 +43861,13 @@
         <v>0</v>
       </c>
       <c r="Z393" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA393" s="3" t="n">
         <v>690</v>
       </c>
       <c r="AB393" s="3" t="n">
-        <v>0</v>
+        <v>1531</v>
       </c>
       <c r="AC393" s="3" t="n">
         <v>26404</v>
@@ -43967,7 +43967,7 @@
         <v>428</v>
       </c>
       <c r="AB394" s="3" t="n">
-        <v>0</v>
+        <v>323</v>
       </c>
       <c r="AC394" s="3" t="n">
         <v>24297</v>
@@ -44067,7 +44067,7 @@
         <v>648</v>
       </c>
       <c r="AB395" s="3" t="n">
-        <v>0</v>
+        <v>357</v>
       </c>
       <c r="AC395" s="3" t="n">
         <v>22037</v>
@@ -44158,16 +44158,16 @@
         <v>0.0009810000000000001</v>
       </c>
       <c r="Y396" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z396" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA396" s="3" t="n">
         <v>562</v>
       </c>
       <c r="AB396" s="3" t="n">
-        <v>0</v>
+        <v>281</v>
       </c>
       <c r="AC396" s="3" t="n">
         <v>24440</v>
@@ -44267,7 +44267,7 @@
         <v>336</v>
       </c>
       <c r="AB397" s="3" t="n">
-        <v>0</v>
+        <v>166</v>
       </c>
       <c r="AC397" s="3" t="n">
         <v>21752</v>
@@ -44367,7 +44367,7 @@
         <v>528</v>
       </c>
       <c r="AB398" s="3" t="n">
-        <v>0</v>
+        <v>204</v>
       </c>
       <c r="AC398" s="3" t="n">
         <v>22479</v>
@@ -44461,13 +44461,13 @@
         <v>0</v>
       </c>
       <c r="Z399" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA399" s="3" t="n">
         <v>506</v>
       </c>
       <c r="AB399" s="3" t="n">
-        <v>0</v>
+        <v>377</v>
       </c>
       <c r="AC399" s="3" t="n">
         <v>20397</v>
@@ -44567,7 +44567,7 @@
         <v>643</v>
       </c>
       <c r="AB400" s="3" t="n">
-        <v>0</v>
+        <v>276</v>
       </c>
       <c r="AC400" s="3" t="n">
         <v>15729</v>
@@ -44667,7 +44667,7 @@
         <v>1387</v>
       </c>
       <c r="AB401" s="3" t="n">
-        <v>0</v>
+        <v>1804</v>
       </c>
       <c r="AC401" s="3" t="n">
         <v>28979</v>
@@ -44708,7 +44708,7 @@
         <v>0.797651</v>
       </c>
       <c r="AB402" s="3" t="n">
-        <v>0.139452</v>
+        <v>0.737333</v>
       </c>
       <c r="AC402" s="3" t="n">
         <v>0.940313</v>
@@ -44740,16 +44740,16 @@
         <v>0.58377</v>
       </c>
       <c r="Y403" s="3" t="n">
-        <v>0.108655</v>
+        <v>0.126771</v>
       </c>
       <c r="Z403" s="3" t="n">
-        <v>0.13215</v>
+        <v>0.127874</v>
       </c>
       <c r="AA403" s="3" t="n">
         <v>0.6093150000000001</v>
       </c>
       <c r="AB403" s="3" t="n">
-        <v>0.16775</v>
+        <v>0.498466</v>
       </c>
       <c r="AC403" s="3" t="n">
         <v>0.830507</v>
@@ -44774,20 +44774,20 @@
       </c>
       <c r="W404" s="3" t="inlineStr">
         <is>
-          <t>pearson  (*,  EV)</t>
+          <t>pearson  (*,  NV)</t>
         </is>
       </c>
       <c r="X404" s="3" t="n">
-        <v>0.148412</v>
+        <v>0.7063199999999999</v>
       </c>
       <c r="Y404" s="3" t="n">
-        <v>-0.005699</v>
+        <v>0.733924</v>
       </c>
       <c r="Z404" s="3" t="n">
-        <v>-0.005617</v>
-      </c>
-      <c r="AA404" s="3" t="n">
-        <v>0.797651</v>
+        <v>0.733855</v>
+      </c>
+      <c r="AC404" s="3" t="n">
+        <v>0.646591</v>
       </c>
     </row>
     <row r="405">
@@ -44801,20 +44801,17 @@
       </c>
       <c r="W405" s="3" t="inlineStr">
         <is>
-          <t>spearman (*,  EV)</t>
+          <t>spearman (*,  NV)</t>
         </is>
       </c>
       <c r="X405" s="3" t="n">
-        <v>0.160764</v>
+        <v>0.460874</v>
       </c>
       <c r="Y405" s="3" t="n">
-        <v>0.232399</v>
+        <v>0.314408</v>
       </c>
       <c r="Z405" s="3" t="n">
-        <v>0.230312</v>
-      </c>
-      <c r="AA405" s="3" t="n">
-        <v>0.6093150000000001</v>
+        <v>0.305723</v>
       </c>
     </row>
     <row r="406">
@@ -44840,9 +44837,6 @@
       <c r="Z406" s="3" t="n">
         <v>0.649384</v>
       </c>
-      <c r="AC406" s="3" t="n">
-        <v>0.940313</v>
-      </c>
     </row>
     <row r="407">
       <c r="H407" s="3" t="inlineStr">
@@ -44862,13 +44856,10 @@
         <v>0.810408</v>
       </c>
       <c r="Y407" s="3" t="n">
-        <v>-0.104138</v>
+        <v>-0.065946</v>
       </c>
       <c r="Z407" s="3" t="n">
-        <v>-0.090526</v>
-      </c>
-      <c r="AC407" s="3" t="n">
-        <v>0.830507</v>
+        <v>-0.072004</v>
       </c>
     </row>
     <row r="408">
@@ -44881,13 +44872,10 @@
         <v>0.624937</v>
       </c>
       <c r="Y408" s="3" t="n">
-        <v>-0.070451</v>
+        <v>-0.04208</v>
       </c>
       <c r="Z408" s="3" t="n">
-        <v>-0.060777</v>
-      </c>
-      <c r="AC408" s="3" t="n">
-        <v>0.646591</v>
+        <v>-0.046892</v>
       </c>
     </row>
     <row r="409">
@@ -44913,7 +44901,7 @@
       </c>
       <c r="AB409" s="1" t="inlineStr">
         <is>
-          <t>EpiRank (EV)</t>
+          <t>EpiRank (NV)</t>
         </is>
       </c>
       <c r="AC409" s="1" t="inlineStr">
@@ -45026,26 +45014,26 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>EV</t>
+          <t>NV</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.139452</v>
+        <v>0.737333</v>
       </c>
       <c r="D3" t="n">
-        <v>0.16775</v>
+        <v>0.498466</v>
       </c>
       <c r="E3" t="n">
-        <v>0.136574</v>
+        <v>0.345938</v>
       </c>
       <c r="F3" t="n">
-        <v>0.8181818181818182</v>
+        <v>0.5886524822695035</v>
       </c>
       <c r="G3" t="n">
-        <v>0.06382978723404255</v>
+        <v>0.5886524822695035</v>
       </c>
       <c r="H3" t="n">
-        <v>0.1184210526315789</v>
+        <v>0.5886524822695035</v>
       </c>
     </row>
     <row r="4">
@@ -45116,26 +45104,26 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>EV</t>
+          <t>NV</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.148412</v>
+        <v>0.7063199999999999</v>
       </c>
       <c r="D6" t="n">
-        <v>0.160764</v>
+        <v>0.460874</v>
       </c>
       <c r="E6" t="n">
-        <v>0.130657</v>
+        <v>0.318464</v>
       </c>
       <c r="F6" t="n">
-        <v>0.6363636363636364</v>
+        <v>0.5390070921985816</v>
       </c>
       <c r="G6" t="n">
-        <v>0.05426356589147287</v>
+        <v>0.5891472868217055</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1</v>
+        <v>0.5629629629629629</v>
       </c>
     </row>
     <row r="7">
@@ -45183,10 +45171,10 @@
         <v>0.467527</v>
       </c>
       <c r="D8" t="n">
-        <v>0.108655</v>
+        <v>0.126771</v>
       </c>
       <c r="E8" t="n">
-        <v>0.067755</v>
+        <v>0.08189200000000001</v>
       </c>
       <c r="F8" t="n">
         <v/>
@@ -45206,17 +45194,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>EV</t>
+          <t>NV</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>-0.005699</v>
+        <v>0.733924</v>
       </c>
       <c r="D9" t="n">
-        <v>0.232399</v>
+        <v>0.314408</v>
       </c>
       <c r="E9" t="n">
-        <v>0.190041</v>
+        <v>0.211273</v>
       </c>
       <c r="F9" t="n">
         <v/>
@@ -45243,10 +45231,10 @@
         <v>0.649212</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.104138</v>
+        <v>-0.065946</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.070451</v>
+        <v>-0.04208</v>
       </c>
       <c r="F10" t="n">
         <v/>
@@ -45273,10 +45261,10 @@
         <v>0.467574</v>
       </c>
       <c r="D11" t="n">
-        <v>0.13215</v>
+        <v>0.127874</v>
       </c>
       <c r="E11" t="n">
-        <v>0.087006</v>
+        <v>0.082469</v>
       </c>
       <c r="F11" t="n">
         <v/>
@@ -45296,17 +45284,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>EV</t>
+          <t>NV</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>-0.005617</v>
+        <v>0.733855</v>
       </c>
       <c r="D12" t="n">
-        <v>0.230312</v>
+        <v>0.305723</v>
       </c>
       <c r="E12" t="n">
-        <v>0.188428</v>
+        <v>0.204404</v>
       </c>
       <c r="F12" t="n">
         <v/>
@@ -45333,10 +45321,10 @@
         <v>0.649384</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.090526</v>
+        <v>-0.072004</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.060777</v>
+        <v>-0.046892</v>
       </c>
       <c r="F13" t="n">
         <v/>
@@ -45386,26 +45374,26 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>EV</t>
+          <t>NV</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.10581</v>
+        <v>0.837454</v>
       </c>
       <c r="D15" t="n">
-        <v>0.191381</v>
+        <v>0.633255</v>
       </c>
       <c r="E15" t="n">
-        <v>0.156261</v>
+        <v>0.459697</v>
       </c>
       <c r="F15" t="n">
-        <v>0.9090909090909091</v>
+        <v>0.6312056737588653</v>
       </c>
       <c r="G15" t="n">
-        <v>0.07633587786259542</v>
+        <v>0.6793893129770993</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1408450704225352</v>
+        <v>0.6544117647058824</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(epirank): refresh ERA results (3 json + 3 xlsx) after latest run
</commit_message>
<xml_diff>
--- a/EpiRank_原_Germany/ERA_result_d_0.95_daytime_0.5_loops_110.xlsx
+++ b/EpiRank_原_Germany/ERA_result_d_0.95_daytime_0.5_loops_110.xlsx
@@ -859,10 +859,10 @@
         <v>0.019464</v>
       </c>
       <c r="Y3" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z3" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA3" s="3" t="n">
         <v>34035</v>
@@ -1435,7 +1435,7 @@
         <v>0.01118</v>
       </c>
       <c r="Y7" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z7" s="3" t="n">
         <v>-0</v>
@@ -2148,10 +2148,10 @@
         <v>0.007346</v>
       </c>
       <c r="Y12" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z12" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA12" s="3" t="n">
         <v>6490</v>
@@ -2293,10 +2293,10 @@
         <v>0.005667</v>
       </c>
       <c r="Y13" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z13" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA13" s="3" t="n">
         <v>1620</v>
@@ -2558,10 +2558,10 @@
         <v>0.005871</v>
       </c>
       <c r="Y15" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z15" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA15" s="3" t="n">
         <v>4465</v>
@@ -2941,7 +2941,7 @@
         <v>0</v>
       </c>
       <c r="Z18" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA18" s="3" t="n">
         <v>2380</v>
@@ -3418,10 +3418,10 @@
         <v>0.004559</v>
       </c>
       <c r="Y22" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z22" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA22" s="3" t="n">
         <v>4123</v>
@@ -3778,10 +3778,10 @@
         <v>0.004167</v>
       </c>
       <c r="Y25" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z25" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA25" s="3" t="n">
         <v>3606</v>
@@ -4018,7 +4018,7 @@
         <v>0.004805</v>
       </c>
       <c r="Y27" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z27" s="3" t="n">
         <v>0</v>
@@ -4378,10 +4378,10 @@
         <v>0.004758</v>
       </c>
       <c r="Y30" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z30" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA30" s="3" t="n">
         <v>2551</v>
@@ -4978,10 +4978,10 @@
         <v>0.004087</v>
       </c>
       <c r="Y35" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z35" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA35" s="3" t="n">
         <v>2538</v>
@@ -5098,7 +5098,7 @@
         <v>0.003865</v>
       </c>
       <c r="Y36" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z36" s="3" t="n">
         <v>-0</v>
@@ -5221,7 +5221,7 @@
         <v>0</v>
       </c>
       <c r="Z37" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA37" s="3" t="n">
         <v>2678</v>
@@ -5818,10 +5818,10 @@
         <v>0.003867</v>
       </c>
       <c r="Y42" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z42" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA42" s="3" t="n">
         <v>3417</v>
@@ -5941,7 +5941,7 @@
         <v>0</v>
       </c>
       <c r="Z43" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA43" s="3" t="n">
         <v>2060</v>
@@ -6058,10 +6058,10 @@
         <v>0.003516</v>
       </c>
       <c r="Y44" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z44" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA44" s="3" t="n">
         <v>2752</v>
@@ -6658,7 +6658,7 @@
         <v>0.003683</v>
       </c>
       <c r="Y49" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z49" s="3" t="n">
         <v>-0</v>
@@ -7618,10 +7618,10 @@
         <v>0.003258</v>
       </c>
       <c r="Y57" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z57" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA57" s="3" t="n">
         <v>1293</v>
@@ -8698,10 +8698,10 @@
         <v>0.002932</v>
       </c>
       <c r="Y66" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z66" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA66" s="3" t="n">
         <v>2443</v>
@@ -9778,10 +9778,10 @@
         <v>0.003381</v>
       </c>
       <c r="Y75" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z75" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA75" s="3" t="n">
         <v>1306</v>
@@ -10258,7 +10258,7 @@
         <v>0.002994</v>
       </c>
       <c r="Y79" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z79" s="3" t="n">
         <v>-0</v>
@@ -11458,7 +11458,7 @@
         <v>0.002894</v>
       </c>
       <c r="Y89" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z89" s="3" t="n">
         <v>0</v>
@@ -11941,7 +11941,7 @@
         <v>0</v>
       </c>
       <c r="Z93" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA93" s="3" t="n">
         <v>3690</v>
@@ -12658,10 +12658,10 @@
         <v>0.002802</v>
       </c>
       <c r="Y99" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z99" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA99" s="3" t="n">
         <v>2203</v>
@@ -12901,7 +12901,7 @@
         <v>0</v>
       </c>
       <c r="Z101" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA101" s="3" t="n">
         <v>1745</v>
@@ -13018,10 +13018,10 @@
         <v>0.003001</v>
       </c>
       <c r="Y102" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z102" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA102" s="3" t="n">
         <v>3835</v>
@@ -13378,10 +13378,10 @@
         <v>0.002646</v>
       </c>
       <c r="Y105" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z105" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA105" s="3" t="n">
         <v>4116</v>
@@ -13498,7 +13498,7 @@
         <v>0.002503</v>
       </c>
       <c r="Y106" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z106" s="3" t="n">
         <v>0</v>
@@ -13858,10 +13858,10 @@
         <v>0.002608</v>
       </c>
       <c r="Y109" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z109" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA109" s="3" t="n">
         <v>3508</v>
@@ -13978,10 +13978,10 @@
         <v>0.002646</v>
       </c>
       <c r="Y110" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z110" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA110" s="3" t="n">
         <v>2711</v>
@@ -14698,10 +14698,10 @@
         <v>0.003037</v>
       </c>
       <c r="Y116" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z116" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA116" s="3" t="n">
         <v>2287</v>
@@ -15701,7 +15701,7 @@
         <v>-0</v>
       </c>
       <c r="Z125" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA125" s="3" t="n">
         <v>1517</v>
@@ -15808,10 +15808,10 @@
         <v>0.002434</v>
       </c>
       <c r="Y126" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z126" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA126" s="3" t="n">
         <v>1796</v>
@@ -16358,10 +16358,10 @@
         <v>0.002399</v>
       </c>
       <c r="Y131" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z131" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA131" s="3" t="n">
         <v>2916</v>
@@ -16581,7 +16581,7 @@
         <v>0</v>
       </c>
       <c r="Z133" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA133" s="3" t="n">
         <v>1776</v>
@@ -16908,7 +16908,7 @@
         <v>0.002515</v>
       </c>
       <c r="Y136" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z136" s="3" t="n">
         <v>0</v>
@@ -17128,10 +17128,10 @@
         <v>0.002078</v>
       </c>
       <c r="Y138" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z138" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA138" s="3" t="n">
         <v>1844</v>
@@ -17678,10 +17678,10 @@
         <v>0.002517</v>
       </c>
       <c r="Y143" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z143" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA143" s="3" t="n">
         <v>4137</v>
@@ -18121,7 +18121,7 @@
         <v>0</v>
       </c>
       <c r="Z147" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA147" s="3" t="n">
         <v>2616</v>
@@ -18668,10 +18668,10 @@
         <v>0.002351</v>
       </c>
       <c r="Y152" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z152" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA152" s="3" t="n">
         <v>1967</v>
@@ -19218,10 +19218,10 @@
         <v>0.002359</v>
       </c>
       <c r="Y157" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z157" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA157" s="3" t="n">
         <v>1949</v>
@@ -19551,7 +19551,7 @@
         <v>0</v>
       </c>
       <c r="Z160" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA160" s="3" t="n">
         <v>3546</v>
@@ -19771,7 +19771,7 @@
         <v>-0</v>
       </c>
       <c r="Z162" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA162" s="3" t="n">
         <v>1727</v>
@@ -20098,7 +20098,7 @@
         <v>0.002271</v>
       </c>
       <c r="Y165" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z165" s="3" t="n">
         <v>-0</v>
@@ -20208,10 +20208,10 @@
         <v>0.002226</v>
       </c>
       <c r="Y166" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z166" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA166" s="3" t="n">
         <v>2856</v>
@@ -20761,7 +20761,7 @@
         <v>0</v>
       </c>
       <c r="Z171" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA171" s="3" t="n">
         <v>1737</v>
@@ -21308,10 +21308,10 @@
         <v>0.001886</v>
       </c>
       <c r="Y176" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z176" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA176" s="3" t="n">
         <v>1626</v>
@@ -22411,7 +22411,7 @@
         <v>0</v>
       </c>
       <c r="Z186" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA186" s="3" t="n">
         <v>1460</v>
@@ -22628,10 +22628,10 @@
         <v>0.002033</v>
       </c>
       <c r="Y188" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z188" s="3" t="n">
         <v>-0</v>
-      </c>
-      <c r="Z188" s="3" t="n">
-        <v>0</v>
       </c>
       <c r="AA188" s="3" t="n">
         <v>1846</v>
@@ -24061,7 +24061,7 @@
         <v>0</v>
       </c>
       <c r="Z201" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA201" s="3" t="n">
         <v>1413</v>
@@ -24718,7 +24718,7 @@
         <v>0.001965</v>
       </c>
       <c r="Y207" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z207" s="3" t="n">
         <v>0</v>
@@ -24938,10 +24938,10 @@
         <v>0.001847</v>
       </c>
       <c r="Y209" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z209" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA209" s="3" t="n">
         <v>1086</v>
@@ -25051,7 +25051,7 @@
         <v>0</v>
       </c>
       <c r="Z210" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA210" s="3" t="n">
         <v>1407</v>
@@ -25158,10 +25158,10 @@
         <v>0.001842</v>
       </c>
       <c r="Y211" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z211" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA211" s="3" t="n">
         <v>1124</v>
@@ -25268,7 +25268,7 @@
         <v>0.002032</v>
       </c>
       <c r="Y212" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z212" s="3" t="n">
         <v>-0</v>
@@ -25378,10 +25378,10 @@
         <v>0.00183</v>
       </c>
       <c r="Y213" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z213" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA213" s="3" t="n">
         <v>1611</v>
@@ -25488,10 +25488,10 @@
         <v>0.001952</v>
       </c>
       <c r="Y214" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z214" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA214" s="3" t="n">
         <v>952</v>
@@ -27248,7 +27248,7 @@
         <v>0.001956</v>
       </c>
       <c r="Y230" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z230" s="3" t="n">
         <v>0</v>
@@ -27688,10 +27688,10 @@
         <v>0.001896</v>
       </c>
       <c r="Y234" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z234" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA234" s="3" t="n">
         <v>941</v>
@@ -27801,7 +27801,7 @@
         <v>0</v>
       </c>
       <c r="Z235" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA235" s="3" t="n">
         <v>2347</v>
@@ -28128,10 +28128,10 @@
         <v>0.001669</v>
       </c>
       <c r="Y238" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z238" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA238" s="3" t="n">
         <v>870</v>
@@ -28348,10 +28348,10 @@
         <v>0.001717</v>
       </c>
       <c r="Y240" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z240" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA240" s="3" t="n">
         <v>1789</v>
@@ -28901,7 +28901,7 @@
         <v>-0</v>
       </c>
       <c r="Z245" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA245" s="3" t="n">
         <v>552</v>
@@ -29228,10 +29228,10 @@
         <v>0.001997</v>
       </c>
       <c r="Y248" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z248" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA248" s="3" t="n">
         <v>1537</v>
@@ -29778,10 +29778,10 @@
         <v>0.001785</v>
       </c>
       <c r="Y253" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z253" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA253" s="3" t="n">
         <v>1929</v>
@@ -31158,10 +31158,10 @@
         <v>0.001815</v>
       </c>
       <c r="Y266" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z266" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA266" s="3" t="n">
         <v>1523</v>
@@ -31258,10 +31258,10 @@
         <v>0.001619</v>
       </c>
       <c r="Y267" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z267" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA267" s="3" t="n">
         <v>916</v>
@@ -31958,10 +31958,10 @@
         <v>0.001683</v>
       </c>
       <c r="Y274" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z274" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA274" s="3" t="n">
         <v>3118</v>
@@ -32461,7 +32461,7 @@
         <v>0</v>
       </c>
       <c r="Z279" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA279" s="3" t="n">
         <v>1102</v>
@@ -32558,7 +32558,7 @@
         <v>0.001707</v>
       </c>
       <c r="Y280" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z280" s="3" t="n">
         <v>0</v>
@@ -32758,10 +32758,10 @@
         <v>0.001666</v>
       </c>
       <c r="Y282" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z282" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA282" s="3" t="n">
         <v>2005</v>
@@ -33158,10 +33158,10 @@
         <v>0.001605</v>
       </c>
       <c r="Y286" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z286" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA286" s="3" t="n">
         <v>627</v>
@@ -33258,10 +33258,10 @@
         <v>0.00163</v>
       </c>
       <c r="Y287" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z287" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA287" s="3" t="n">
         <v>2337</v>
@@ -33458,10 +33458,10 @@
         <v>0.001646</v>
       </c>
       <c r="Y289" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z289" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA289" s="3" t="n">
         <v>3450</v>
@@ -34158,7 +34158,7 @@
         <v>0.001582</v>
       </c>
       <c r="Y296" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z296" s="3" t="n">
         <v>0</v>
@@ -35558,7 +35558,7 @@
         <v>0.00142</v>
       </c>
       <c r="Y310" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z310" s="3" t="n">
         <v>0</v>
@@ -36061,7 +36061,7 @@
         <v>0</v>
       </c>
       <c r="Z315" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA315" s="3" t="n">
         <v>1537</v>
@@ -36361,7 +36361,7 @@
         <v>0</v>
       </c>
       <c r="Z318" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA318" s="3" t="n">
         <v>800</v>
@@ -36858,7 +36858,7 @@
         <v>0.001535</v>
       </c>
       <c r="Y323" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z323" s="3" t="n">
         <v>-0</v>
@@ -37061,7 +37061,7 @@
         <v>0</v>
       </c>
       <c r="Z325" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA325" s="3" t="n">
         <v>953</v>
@@ -37258,10 +37258,10 @@
         <v>0.001423</v>
       </c>
       <c r="Y327" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z327" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA327" s="3" t="n">
         <v>481</v>
@@ -37361,7 +37361,7 @@
         <v>0</v>
       </c>
       <c r="Z328" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA328" s="3" t="n">
         <v>2839</v>
@@ -37558,10 +37558,10 @@
         <v>0.001302</v>
       </c>
       <c r="Y330" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z330" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA330" s="3" t="n">
         <v>849</v>
@@ -39258,10 +39258,10 @@
         <v>0.001345</v>
       </c>
       <c r="Y347" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z347" s="3" t="n">
         <v>-0</v>
-      </c>
-      <c r="Z347" s="3" t="n">
-        <v>0</v>
       </c>
       <c r="AA347" s="3" t="n">
         <v>1161</v>
@@ -39361,7 +39361,7 @@
         <v>0</v>
       </c>
       <c r="Z348" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA348" s="3" t="n">
         <v>1209</v>
@@ -39761,7 +39761,7 @@
         <v>0</v>
       </c>
       <c r="Z352" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA352" s="3" t="n">
         <v>2349</v>
@@ -40458,10 +40458,10 @@
         <v>0.00144</v>
       </c>
       <c r="Y359" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z359" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA359" s="3" t="n">
         <v>622</v>
@@ -42058,10 +42058,10 @@
         <v>0.000982</v>
       </c>
       <c r="Y375" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z375" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA375" s="3" t="n">
         <v>1642</v>
@@ -42358,10 +42358,10 @@
         <v>0.001213</v>
       </c>
       <c r="Y378" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z378" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA378" s="3" t="n">
         <v>343</v>
@@ -42661,7 +42661,7 @@
         <v>0</v>
       </c>
       <c r="Z381" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA381" s="3" t="n">
         <v>330</v>
@@ -42761,7 +42761,7 @@
         <v>0</v>
       </c>
       <c r="Z382" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA382" s="3" t="n">
         <v>1161</v>
@@ -42858,10 +42858,10 @@
         <v>0.001105</v>
       </c>
       <c r="Y383" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z383" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA383" s="3" t="n">
         <v>247</v>
@@ -42958,10 +42958,10 @@
         <v>0.001039</v>
       </c>
       <c r="Y384" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z384" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA384" s="3" t="n">
         <v>242</v>
@@ -43861,7 +43861,7 @@
         <v>0</v>
       </c>
       <c r="Z393" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA393" s="3" t="n">
         <v>690</v>
@@ -44058,10 +44058,10 @@
         <v>0.00096</v>
       </c>
       <c r="Y395" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z395" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA395" s="3" t="n">
         <v>648</v>
@@ -44158,7 +44158,7 @@
         <v>0.0009810000000000001</v>
       </c>
       <c r="Y396" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z396" s="3" t="n">
         <v>-0</v>
@@ -44558,10 +44558,10 @@
         <v>0.000806</v>
       </c>
       <c r="Y400" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z400" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA400" s="3" t="n">
         <v>643</v>
@@ -44707,12 +44707,6 @@
       <c r="AA402" s="3" t="n">
         <v>0.797651</v>
       </c>
-      <c r="AB402" s="3" t="n">
-        <v>0.737333</v>
-      </c>
-      <c r="AC402" s="3" t="n">
-        <v>0.940313</v>
-      </c>
     </row>
     <row r="403">
       <c r="H403" s="3" t="inlineStr">
@@ -44740,19 +44734,13 @@
         <v>0.58377</v>
       </c>
       <c r="Y403" s="3" t="n">
-        <v>0.126771</v>
+        <v>0.162933</v>
       </c>
       <c r="Z403" s="3" t="n">
-        <v>0.127874</v>
+        <v>0.135769</v>
       </c>
       <c r="AA403" s="3" t="n">
         <v>0.6093150000000001</v>
-      </c>
-      <c r="AB403" s="3" t="n">
-        <v>0.498466</v>
-      </c>
-      <c r="AC403" s="3" t="n">
-        <v>0.830507</v>
       </c>
     </row>
     <row r="404">
@@ -44786,8 +44774,8 @@
       <c r="Z404" s="3" t="n">
         <v>0.733855</v>
       </c>
-      <c r="AC404" s="3" t="n">
-        <v>0.646591</v>
+      <c r="AB404" s="3" t="n">
+        <v>0.737333</v>
       </c>
     </row>
     <row r="405">
@@ -44808,10 +44796,13 @@
         <v>0.460874</v>
       </c>
       <c r="Y405" s="3" t="n">
-        <v>0.314408</v>
+        <v>0.310688</v>
       </c>
       <c r="Z405" s="3" t="n">
-        <v>0.305723</v>
+        <v>0.284487</v>
+      </c>
+      <c r="AB405" s="3" t="n">
+        <v>0.498466</v>
       </c>
     </row>
     <row r="406">
@@ -44837,6 +44828,9 @@
       <c r="Z406" s="3" t="n">
         <v>0.649384</v>
       </c>
+      <c r="AC406" s="3" t="n">
+        <v>0.940313</v>
+      </c>
     </row>
     <row r="407">
       <c r="H407" s="3" t="inlineStr">
@@ -44856,10 +44850,13 @@
         <v>0.810408</v>
       </c>
       <c r="Y407" s="3" t="n">
-        <v>-0.065946</v>
+        <v>-0.056118</v>
       </c>
       <c r="Z407" s="3" t="n">
-        <v>-0.072004</v>
+        <v>-0.095414</v>
+      </c>
+      <c r="AC407" s="3" t="n">
+        <v>0.830507</v>
       </c>
     </row>
     <row r="408">
@@ -44872,10 +44869,13 @@
         <v>0.624937</v>
       </c>
       <c r="Y408" s="3" t="n">
-        <v>-0.04208</v>
+        <v>-0.035915</v>
       </c>
       <c r="Z408" s="3" t="n">
-        <v>-0.046892</v>
+        <v>-0.063609</v>
+      </c>
+      <c r="AC408" s="3" t="n">
+        <v>0.646591</v>
       </c>
     </row>
     <row r="409">
@@ -45171,10 +45171,10 @@
         <v>0.467527</v>
       </c>
       <c r="D8" t="n">
-        <v>0.126771</v>
+        <v>0.162933</v>
       </c>
       <c r="E8" t="n">
-        <v>0.08189200000000001</v>
+        <v>0.110192</v>
       </c>
       <c r="F8" t="n">
         <v/>
@@ -45201,10 +45201,10 @@
         <v>0.733924</v>
       </c>
       <c r="D9" t="n">
-        <v>0.314408</v>
+        <v>0.310688</v>
       </c>
       <c r="E9" t="n">
-        <v>0.211273</v>
+        <v>0.205683</v>
       </c>
       <c r="F9" t="n">
         <v/>
@@ -45231,10 +45231,10 @@
         <v>0.649212</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.065946</v>
+        <v>-0.056118</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.04208</v>
+        <v>-0.035915</v>
       </c>
       <c r="F10" t="n">
         <v/>
@@ -45261,10 +45261,10 @@
         <v>0.467574</v>
       </c>
       <c r="D11" t="n">
-        <v>0.127874</v>
+        <v>0.135769</v>
       </c>
       <c r="E11" t="n">
-        <v>0.082469</v>
+        <v>0.088986</v>
       </c>
       <c r="F11" t="n">
         <v/>
@@ -45291,10 +45291,10 @@
         <v>0.733855</v>
       </c>
       <c r="D12" t="n">
-        <v>0.305723</v>
+        <v>0.284487</v>
       </c>
       <c r="E12" t="n">
-        <v>0.204404</v>
+        <v>0.186055</v>
       </c>
       <c r="F12" t="n">
         <v/>
@@ -45321,10 +45321,10 @@
         <v>0.649384</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.072004</v>
+        <v>-0.095414</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.046892</v>
+        <v>-0.063609</v>
       </c>
       <c r="F13" t="n">
         <v/>

</xml_diff>